<commit_message>
Cập nhật skill và tài liệu plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrm/.plans/gop-db/warranty-repair-handle-request/testcase.xlsx
+++ b/hrm/.plans/gop-db/warranty-repair-handle-request/testcase.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q116"/>
+  <dimension ref="A1:Q121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26.9" customWidth="1" min="1" max="1"/>
@@ -847,7 +847,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Testcase _ Phiếu xử lý yêu cầu - Cập nhật ngày 21/08/2026</t>
+          <t>Testcase _ Phiếu xử lý yêu cầu - Cập nhật ngày 03/09/2026</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -3626,30 +3626,77 @@
       <c r="P57" s="16" t="inlineStr"/>
       <c r="Q57" s="16" t="inlineStr"/>
     </row>
-    <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="13" t="n"/>
-      <c r="B58" s="13" t="n"/>
-      <c r="C58" s="14" t="inlineStr">
-        <is>
-          <t>IV. LẬP PHIẾU, SỬA &amp; XEM</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="n"/>
-      <c r="E58" s="4" t="n"/>
-      <c r="F58" s="4" t="n"/>
-      <c r="G58" s="4" t="n"/>
-      <c r="H58" s="4" t="n"/>
-      <c r="I58" s="4" t="n"/>
-      <c r="J58" s="4" t="n"/>
-      <c r="K58" s="4" t="n"/>
-      <c r="L58" s="4" t="n"/>
-      <c r="M58" s="4" t="n"/>
-      <c r="N58" s="4" t="n"/>
-      <c r="O58" s="4" t="n"/>
-      <c r="P58" s="4" t="n"/>
-      <c r="Q58" s="5" t="n"/>
-    </row>
-    <row r="59" ht="80" customHeight="1">
+    <row r="58" ht="45" customHeight="1">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>DANH SÁCH, SẮP XẾP &amp; PHÂN TRANG</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>TC_03.005</t>
+        </is>
+      </c>
+      <c r="D58" s="15" t="inlineStr">
+        <is>
+          <t>Bật cột Người cập nhật / Ngày cập nhật</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>Có 1 phiếu vừa được sửa lại sau khi lập.</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Cấu hình cột hiển thị
+2. Bật Người cập nhật và Ngày cập nhật
+3. Lưu lại</t>
+        </is>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
+        <is>
+          <t>Bật: Người cập nhật, Ngày cập nhật</t>
+        </is>
+      </c>
+      <c r="I58" s="15" t="inlineStr">
+        <is>
+          <t>- Hai cột hiện ở cuối bảng, đúng người sửa gần nhất và đúng thời điểm
+- Phiếu chưa ai sửa lại thì 2 ô này để trống, không hiện ký tự lạ</t>
+        </is>
+      </c>
+      <c r="J58" s="15" t="inlineStr"/>
+      <c r="K58" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L58" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N58" s="15" t="inlineStr"/>
+      <c r="O58" s="16" t="inlineStr"/>
+      <c r="P58" s="16" t="inlineStr"/>
+      <c r="Q58" s="16" t="inlineStr"/>
+    </row>
+    <row r="59" ht="42" customHeight="1">
       <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -3657,33 +3704,33 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
+          <t>DANH SÁCH, SẮP XẾP &amp; PHÂN TRANG</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>TC_04.001</t>
+          <t>TC_03.006</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>Lập phiếu xử lý từ Phiếu yêu cầu</t>
+          <t>Cột Ngày xử lý chỉ có khi đã lập phiếu cung cấp thông tin</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F59" s="15" t="inlineStr">
         <is>
-          <t>Phiếu yêu cầu Y đang “Chờ xử lý”, gửi về phòng của người đăng nhập, chưa có phiếu xử lý nào.</t>
+          <t>Có 1 phiếu ở “Chờ CCTT” và 1 phiếu ở “Đã CCTT”.</t>
         </is>
       </c>
       <c r="G59" s="15" t="inlineStr">
         <is>
-          <t>1. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành
-2. Ở dòng phiếu Y, bấm “Tạo phiếu xử lý yêu cầu”</t>
+          <t>1. Bật cột Ngày xử lý
+2. So 2 phiếu</t>
         </is>
       </c>
       <c r="H59" s="15" t="inlineStr">
@@ -3693,9 +3740,8 @@
       </c>
       <c r="I59" s="15" t="inlineStr">
         <is>
-          <t>- Mở màn “Lập phiếu xử lý yêu cầu”
-- Khối Thông tin yêu cầu điền sẵn và KHÓA: Phiếu yêu cầu, Người yêu cầu, Phòng yêu cầu, Ngày nhận yêu cầu, Khách hàng, Người liên hệ, SĐT, Địa chỉ sửa chữa
-- Bảng thiết bị chép đủ số dòng của phiếu yêu cầu</t>
+          <t>- Phiếu “Đã CCTT” có Ngày xử lý
+- ⚠️ Phiếu “Chờ CCTT” để trống — mốc này do màn Phiếu cung cấp thông tin ghi, không phải màn này</t>
         </is>
       </c>
       <c r="J59" s="15" t="inlineStr"/>
@@ -3719,120 +3765,76 @@
       <c r="P59" s="16" t="inlineStr"/>
       <c r="Q59" s="16" t="inlineStr"/>
     </row>
-    <row r="60" ht="46" customHeight="1">
-      <c r="A60" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B60" s="15" t="inlineStr">
+    <row r="60" ht="26" customHeight="1">
+      <c r="A60" s="13" t="n"/>
+      <c r="B60" s="13" t="n"/>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>IV. LẬP PHIẾU, SỬA &amp; XEM</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n"/>
+      <c r="E60" s="4" t="n"/>
+      <c r="F60" s="4" t="n"/>
+      <c r="G60" s="4" t="n"/>
+      <c r="H60" s="4" t="n"/>
+      <c r="I60" s="4" t="n"/>
+      <c r="J60" s="4" t="n"/>
+      <c r="K60" s="4" t="n"/>
+      <c r="L60" s="4" t="n"/>
+      <c r="M60" s="4" t="n"/>
+      <c r="N60" s="4" t="n"/>
+      <c r="O60" s="4" t="n"/>
+      <c r="P60" s="4" t="n"/>
+      <c r="Q60" s="5" t="n"/>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>LẬP PHIẾU, SỬA &amp; XEM</t>
         </is>
       </c>
-      <c r="C60" s="16" t="inlineStr">
-        <is>
-          <t>TC_04.002</t>
-        </is>
-      </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>Không lập được phiếu khi phiếu yêu cầu không đủ điều kiện</t>
-        </is>
-      </c>
-      <c r="E60" s="16" t="inlineStr">
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>TC_04.001</t>
+        </is>
+      </c>
+      <c r="D61" s="15" t="inlineStr">
+        <is>
+          <t>Lập phiếu xử lý từ Phiếu yêu cầu</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F60" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu yêu cầu đã có phiếu xử lý; và một phiếu yêu cầu khác đang ở “Đang tạo”.</t>
-        </is>
-      </c>
-      <c r="G60" s="15" t="inlineStr">
-        <is>
-          <t>1. Gõ thẳng đường dẫn màn lập phiếu kèm mã của 2 phiếu yêu cầu trên</t>
-        </is>
-      </c>
-      <c r="H60" s="15" t="inlineStr">
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu yêu cầu Y đang “Chờ xử lý”, gửi về phòng của người đăng nhập, chưa có phiếu xử lý nào.</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>1. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành
+2. Ở dòng phiếu Y, bấm “Tạo phiếu xử lý yêu cầu”</t>
+        </is>
+      </c>
+      <c r="H61" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I60" s="15" t="inlineStr">
-        <is>
-          <t>- Cả 2 lần đều bị từ chối, báo phiếu yêu cầu không ở trạng thái chờ xử lý của phòng bạn hoặc đã có phiếu xử lý
-- Được đưa về màn danh sách</t>
-        </is>
-      </c>
-      <c r="J60" s="15" t="inlineStr"/>
-      <c r="K60" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L60" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M60" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N60" s="15" t="inlineStr"/>
-      <c r="O60" s="16" t="inlineStr"/>
-      <c r="P60" s="16" t="inlineStr"/>
-      <c r="Q60" s="16" t="inlineStr"/>
-    </row>
-    <row r="61" ht="44" customHeight="1">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B61" s="15" t="inlineStr">
-        <is>
-          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
-        </is>
-      </c>
-      <c r="C61" s="16" t="inlineStr">
-        <is>
-          <t>TC_04.003</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
-        <is>
-          <t>Chọn nguyên nhân cho từng thiết bị</t>
-        </is>
-      </c>
-      <c r="E61" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F61" s="15" t="inlineStr">
-        <is>
-          <t>Đang ở màn lập phiếu, hàng hóa của dòng đã khai lỗi trong danh mục.</t>
-        </is>
-      </c>
-      <c r="G61" s="15" t="inlineStr">
-        <is>
-          <t>1. Mở ô Nguyên nhân của dòng thiết bị
-2. Chọn 2 nguyên nhân</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I61" s="15" t="inlineStr">
         <is>
-          <t>- Ô cho chọn NHIỀU nguyên nhân, hiện dạng thẻ
-- ⚠️ Danh sách chỉ gồm lỗi đã khai cho ĐÚNG hàng hóa của dòng đó, không phải cả danh mục</t>
+          <t>- Mở màn “Lập phiếu xử lý yêu cầu”
+- Khối Thông tin yêu cầu điền sẵn và KHÓA: Phiếu yêu cầu, Người yêu cầu, Phòng yêu cầu, Ngày nhận yêu cầu, Khách hàng, Người liên hệ, SĐT, Địa chỉ sửa chữa
+- Bảng thiết bị chép đủ số dòng của phiếu yêu cầu</t>
         </is>
       </c>
       <c r="J61" s="15" t="inlineStr"/>
@@ -3856,7 +3858,7 @@
       <c r="P61" s="16" t="inlineStr"/>
       <c r="Q61" s="16" t="inlineStr"/>
     </row>
-    <row r="62" ht="44" customHeight="1">
+    <row r="62" ht="46" customHeight="1">
       <c r="A62" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -3869,27 +3871,27 @@
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>TC_04.004</t>
+          <t>TC_04.002</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
         <is>
-          <t>Hàng hóa chưa khai lỗi nào</t>
+          <t>Không lập được phiếu khi phiếu yêu cầu không đủ điều kiện</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F62" s="15" t="inlineStr">
         <is>
-          <t>Dòng thiết bị có hàng hóa chưa được khai lỗi trong danh mục.</t>
+          <t>Phiếu yêu cầu đã có phiếu xử lý; và một phiếu yêu cầu khác đang ở “Đang tạo”.</t>
         </is>
       </c>
       <c r="G62" s="15" t="inlineStr">
         <is>
-          <t>1. Mở ô Nguyên nhân của dòng đó</t>
+          <t>1. Gõ thẳng đường dẫn màn lập phiếu kèm mã của 2 phiếu yêu cầu trên</t>
         </is>
       </c>
       <c r="H62" s="15" t="inlineStr">
@@ -3899,9 +3901,8 @@
       </c>
       <c r="I62" s="15" t="inlineStr">
         <is>
-          <t>- Ô không có lựa chọn nào
-- Có dòng chữ xám: “Hàng hóa này chưa khai lỗi thiết bị nào trong danh mục.”
-- Có nút “Thêm nhanh” ngay dưới</t>
+          <t>- Cả 2 lần đều bị từ chối, báo phiếu yêu cầu không ở trạng thái chờ xử lý của phòng bạn hoặc đã có phiếu xử lý
+- Được đưa về màn danh sách</t>
         </is>
       </c>
       <c r="J62" s="15" t="inlineStr"/>
@@ -3925,7 +3926,7 @@
       <c r="P62" s="16" t="inlineStr"/>
       <c r="Q62" s="16" t="inlineStr"/>
     </row>
-    <row r="63" ht="39" customHeight="1">
+    <row r="63" ht="44" customHeight="1">
       <c r="A63" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -3938,12 +3939,12 @@
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>TC_04.005</t>
+          <t>TC_04.003</t>
         </is>
       </c>
       <c r="D63" s="15" t="inlineStr">
         <is>
-          <t>Chọn hành động Cung cấp thông tin làm báo giá</t>
+          <t>Chọn nguyên nhân cho từng thiết bị</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
@@ -3953,12 +3954,13 @@
       </c>
       <c r="F63" s="15" t="inlineStr">
         <is>
-          <t>Đang ở màn lập phiếu, đã chọn nguyên nhân.</t>
+          <t>Đang ở màn lập phiếu, hàng hóa của dòng đã khai lỗi trong danh mục.</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
         <is>
-          <t>1. Mở ô Hành động, chọn “Cung cấp thông tin làm báo giá”</t>
+          <t>1. Mở ô Nguyên nhân của dòng thiết bị
+2. Chọn 2 nguyên nhân</t>
         </is>
       </c>
       <c r="H63" s="15" t="inlineStr">
@@ -3968,8 +3970,8 @@
       </c>
       <c r="I63" s="15" t="inlineStr">
         <is>
-          <t>- Ô Hành động có đúng 2 lựa chọn: Tư vấn điện thoại · Cung cấp thông tin làm báo giá
-- Không hiện ô nhập nội dung xử lý</t>
+          <t>- Ô cho chọn NHIỀU nguyên nhân, hiện dạng thẻ
+- ⚠️ Danh sách chỉ gồm lỗi đã khai cho ĐÚNG hàng hóa của dòng đó, không phải cả danh mục</t>
         </is>
       </c>
       <c r="J63" s="15" t="inlineStr"/>
@@ -3993,7 +3995,7 @@
       <c r="P63" s="16" t="inlineStr"/>
       <c r="Q63" s="16" t="inlineStr"/>
     </row>
-    <row r="64" ht="39" customHeight="1">
+    <row r="64" ht="44" customHeight="1">
       <c r="A64" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4006,27 +4008,27 @@
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>TC_04.006</t>
+          <t>TC_04.004</t>
         </is>
       </c>
       <c r="D64" s="15" t="inlineStr">
         <is>
-          <t>Chọn hành động Tư vấn điện thoại thì hiện ô nội dung xử lý</t>
+          <t>Hàng hóa chưa khai lỗi nào</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F64" s="15" t="inlineStr">
         <is>
-          <t>Đang ở màn lập phiếu.</t>
+          <t>Dòng thiết bị có hàng hóa chưa được khai lỗi trong danh mục.</t>
         </is>
       </c>
       <c r="G64" s="15" t="inlineStr">
         <is>
-          <t>1. Chọn hành động “Tư vấn điện thoại”</t>
+          <t>1. Mở ô Nguyên nhân của dòng đó</t>
         </is>
       </c>
       <c r="H64" s="15" t="inlineStr">
@@ -4036,8 +4038,9 @@
       </c>
       <c r="I64" s="15" t="inlineStr">
         <is>
-          <t>- Hiện thêm ô nhập “Nhập nội dung xử lý” ngay dưới
-- Đổi sang hành động khác thì ô này biến mất và nội dung đã gõ bị bỏ</t>
+          <t>- Ô không có lựa chọn nào
+- Có dòng chữ xám: “Hàng hóa này chưa khai lỗi thiết bị nào trong danh mục.”
+- Có nút “Thêm nhanh” ngay dưới</t>
         </is>
       </c>
       <c r="J64" s="15" t="inlineStr"/>
@@ -4061,7 +4064,7 @@
       <c r="P64" s="16" t="inlineStr"/>
       <c r="Q64" s="16" t="inlineStr"/>
     </row>
-    <row r="65" ht="71" customHeight="1">
+    <row r="65" ht="39" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4074,12 +4077,12 @@
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>TC_04.007</t>
+          <t>TC_04.005</t>
         </is>
       </c>
       <c r="D65" s="15" t="inlineStr">
         <is>
-          <t>Thêm nhanh nguyên nhân ngay trong form</t>
+          <t>Chọn hành động Cung cấp thông tin làm báo giá</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
@@ -4089,26 +4092,23 @@
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>Đang ở màn lập/sửa phiếu, người dùng có quyền quản lý danh mục công việc - lỗi thiết bị.</t>
+          <t>Đang ở màn lập phiếu, đã chọn nguyên nhân.</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm “Thêm nhanh” dưới ô Nguyên nhân
-2. Chọn Loại công việc / lỗi, nhập Tên
-3. Bấm Lưu</t>
+          <t>1. Mở ô Hành động, chọn “Cung cấp thông tin làm báo giá”</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
         <is>
-          <t>Loại: Lỗi đã xác định — Tên: “Bục ống dẫn khí nén”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I65" s="15" t="inlineStr">
         <is>
-          <t>- Popup có các ô: Loại, Tên, Định mức công, Định mức đàm phán giá, VAT, Đơn giá bán, Hệ số công nghệ, Ghi chú
-- Lưu xong popup ĐÓNG lại
-- Lỗi mới xuất hiện trong ô Nguyên nhân của đúng dòng đó và được TỰ TÍCH CHỌN</t>
+          <t>- Ô Hành động có đúng 2 lựa chọn: Tư vấn điện thoại · Cung cấp thông tin làm báo giá
+- Không hiện ô nhập nội dung xử lý</t>
         </is>
       </c>
       <c r="J65" s="15" t="inlineStr"/>
@@ -4132,7 +4132,7 @@
       <c r="P65" s="16" t="inlineStr"/>
       <c r="Q65" s="16" t="inlineStr"/>
     </row>
-    <row r="66" ht="34" customHeight="1">
+    <row r="66" ht="39" customHeight="1">
       <c r="A66" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4145,27 +4145,27 @@
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>TC_04.008</t>
+          <t>TC_04.006</t>
         </is>
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>Thêm nhanh thiếu trường bắt buộc</t>
+          <t>Chọn hành động Tư vấn điện thoại thì hiện ô nội dung xử lý</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F66" s="15" t="inlineStr">
         <is>
-          <t>Popup Thêm nhanh đang mở, chưa nhập gì.</t>
+          <t>Đang ở màn lập phiếu.</t>
         </is>
       </c>
       <c r="G66" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu</t>
+          <t>1. Chọn hành động “Tư vấn điện thoại”</t>
         </is>
       </c>
       <c r="H66" s="15" t="inlineStr">
@@ -4175,8 +4175,8 @@
       </c>
       <c r="I66" s="15" t="inlineStr">
         <is>
-          <t>- Báo lỗi đỏ ngay dưới ô Loại và ô Tên
-- Popup không đóng</t>
+          <t>- Hiện thêm ô nhập “Nhập nội dung xử lý” ngay dưới
+- Đổi sang hành động khác thì ô này biến mất và nội dung đã gõ bị bỏ</t>
         </is>
       </c>
       <c r="J66" s="15" t="inlineStr"/>
@@ -4200,7 +4200,7 @@
       <c r="P66" s="16" t="inlineStr"/>
       <c r="Q66" s="16" t="inlineStr"/>
     </row>
-    <row r="67" ht="57" customHeight="1">
+    <row r="67" ht="71" customHeight="1">
       <c r="A67" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>TC_04.009</t>
+          <t>TC_04.007</t>
         </is>
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>Chọn hàng hóa tương đương cho thiết bị tự gõ</t>
+          <t>Thêm nhanh nguyên nhân ngay trong form</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
@@ -4228,26 +4228,26 @@
       </c>
       <c r="F67" s="15" t="inlineStr">
         <is>
-          <t>Phiếu yêu cầu gốc có dòng thiết bị người dùng tự gõ (chưa gắn hàng hóa trong danh mục).</t>
+          <t>Đang ở màn lập/sửa phiếu, người dùng có quyền quản lý danh mục công việc - lỗi thiết bị.</t>
         </is>
       </c>
       <c r="G67" s="15" t="inlineStr">
         <is>
-          <t>1. Ở dòng đó, bấm “Chọn hàng hóa tương đương”
-2. Tìm và chọn một hàng hóa
-3. Xem lại ô Nguyên nhân</t>
+          <t>1. Bấm “Thêm nhanh” dưới ô Nguyên nhân
+2. Chọn Loại công việc / lỗi, nhập Tên
+3. Bấm Lưu</t>
         </is>
       </c>
       <c r="H67" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Loại: Lỗi đã xác định — Tên: “Bục ống dẫn khí nén”</t>
         </is>
       </c>
       <c r="I67" s="15" t="inlineStr">
         <is>
-          <t>- Popup chọn hàng hóa mở ra, tìm được theo tên/mã/model
-- Chọn xong tên hàng hóa hiện thành dòng phụ “Thiết bị tương đương”
-- Danh sách Nguyên nhân nạp lại theo hàng hóa mới</t>
+          <t>- Popup có các ô: Loại, Tên, Định mức công, Định mức đàm phán giá, VAT, Đơn giá bán, Hệ số công nghệ, Ghi chú
+- Lưu xong popup ĐÓNG lại
+- Lỗi mới xuất hiện trong ô Nguyên nhân của đúng dòng đó và được TỰ TÍCH CHỌN</t>
         </is>
       </c>
       <c r="J67" s="15" t="inlineStr"/>
@@ -4271,7 +4271,7 @@
       <c r="P67" s="16" t="inlineStr"/>
       <c r="Q67" s="16" t="inlineStr"/>
     </row>
-    <row r="68" ht="38" customHeight="1">
+    <row r="68" ht="34" customHeight="1">
       <c r="A68" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4284,12 +4284,12 @@
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>TC_04.010</t>
+          <t>TC_04.008</t>
         </is>
       </c>
       <c r="D68" s="15" t="inlineStr">
         <is>
-          <t>Hiển thị tên thiết bị và thiết bị tương đương</t>
+          <t>Thêm nhanh thiếu trường bắt buộc</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="F68" s="15" t="inlineStr">
         <is>
-          <t>Phiếu có dòng thiết bị đã gắn hàng hóa tương đương.</t>
+          <t>Popup Thêm nhanh đang mở, chưa nhập gì.</t>
         </is>
       </c>
       <c r="G68" s="15" t="inlineStr">
         <is>
-          <t>1. Mở màn chi tiết, xem cột Tên hàng hóa</t>
+          <t>1. Bấm Lưu</t>
         </is>
       </c>
       <c r="H68" s="15" t="inlineStr">
@@ -4314,8 +4314,8 @@
       </c>
       <c r="I68" s="15" t="inlineStr">
         <is>
-          <t>- Dòng đầu là tên thiết bị khách báo
-- Dòng phụ nhỏ màu xám: “Thiết bị tương đương: &lt;tên hàng hóa trong danh mục&gt;”</t>
+          <t>- Báo lỗi đỏ ngay dưới ô Loại và ô Tên
+- Popup không đóng</t>
         </is>
       </c>
       <c r="J68" s="15" t="inlineStr"/>
@@ -4339,7 +4339,7 @@
       <c r="P68" s="16" t="inlineStr"/>
       <c r="Q68" s="16" t="inlineStr"/>
     </row>
-    <row r="69" ht="38" customHeight="1">
+    <row r="69" ht="57" customHeight="1">
       <c r="A69" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4352,39 +4352,41 @@
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>TC_04.011</t>
+          <t>TC_04.009</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>Đính kèm tài liệu cho dòng thiết bị</t>
+          <t>Chọn hàng hóa tương đương cho thiết bị tự gõ</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F69" s="15" t="inlineStr">
         <is>
-          <t>Đang lập/sửa phiếu, có sẵn tệp PDF dưới 20MB.</t>
+          <t>Phiếu yêu cầu gốc có dòng thiết bị người dùng tự gõ (chưa gắn hàng hóa trong danh mục).</t>
         </is>
       </c>
       <c r="G69" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Chọn tệp ở cột File đính kèm
-2. Chờ tải xong</t>
+          <t>1. Ở dòng đó, bấm “Chọn hàng hóa tương đương”
+2. Tìm và chọn một hàng hóa
+3. Xem lại ô Nguyên nhân</t>
         </is>
       </c>
       <c r="H69" s="15" t="inlineStr">
         <is>
-          <t>Tệp: bien-ban.pdf</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I69" s="15" t="inlineStr">
         <is>
-          <t>- Trong lúc tải có báo đang tải lên
-- Xong thì hiện biểu tượng loại tệp, tên tệp và 3 nút Tải xuống / Thay đổi / Xóa</t>
+          <t>- Popup chọn hàng hóa mở ra, tìm được theo tên/mã/model
+- Chọn xong tên hàng hóa hiện thành dòng phụ “Thiết bị tương đương”
+- Danh sách Nguyên nhân nạp lại theo hàng hóa mới</t>
         </is>
       </c>
       <c r="J69" s="15" t="inlineStr"/>
@@ -4408,7 +4410,7 @@
       <c r="P69" s="16" t="inlineStr"/>
       <c r="Q69" s="16" t="inlineStr"/>
     </row>
-    <row r="70" ht="34" customHeight="1">
+    <row r="70" ht="38" customHeight="1">
       <c r="A70" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4421,12 +4423,12 @@
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>TC_04.012</t>
+          <t>TC_04.010</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>Chặn đính kèm tệp sai định dạng</t>
+          <t>Hiển thị tên thiết bị và thiết bị tương đương</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
@@ -4436,23 +4438,23 @@
       </c>
       <c r="F70" s="15" t="inlineStr">
         <is>
-          <t>Có sẵn tệp .txt.</t>
+          <t>Phiếu có dòng thiết bị đã gắn hàng hóa tương đương.</t>
         </is>
       </c>
       <c r="G70" s="15" t="inlineStr">
         <is>
-          <t>1. Chọn tệp .txt ở cột File đính kèm</t>
+          <t>1. Mở màn chi tiết, xem cột Tên hàng hóa</t>
         </is>
       </c>
       <c r="H70" s="15" t="inlineStr">
         <is>
-          <t>Tệp: ghi-chu.txt</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I70" s="15" t="inlineStr">
         <is>
-          <t>- Báo chỉ nhận tệp PDF, ảnh, Word hoặc Excel
-- Không tệp nào được gắn vào dòng</t>
+          <t>- Dòng đầu là tên thiết bị khách báo
+- Dòng phụ nhỏ màu xám: “Thiết bị tương đương: &lt;tên hàng hóa trong danh mục&gt;”</t>
         </is>
       </c>
       <c r="J70" s="15" t="inlineStr"/>
@@ -4476,7 +4478,7 @@
       <c r="P70" s="16" t="inlineStr"/>
       <c r="Q70" s="16" t="inlineStr"/>
     </row>
-    <row r="71" ht="45" customHeight="1">
+    <row r="71" ht="38" customHeight="1">
       <c r="A71" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4489,39 +4491,39 @@
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>TC_04.013</t>
+          <t>TC_04.011</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>Lưu nháp</t>
+          <t>Đính kèm tài liệu cho dòng thiết bị</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F71" s="15" t="inlineStr">
         <is>
-          <t>Đang ở màn lập phiếu, chưa chọn nguyên nhân và hành động.</t>
+          <t>Đang lập/sửa phiếu, có sẵn tệp PDF dưới 20MB.</t>
         </is>
       </c>
       <c r="G71" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu nháp</t>
+          <t>1. Bấm Chọn tệp ở cột File đính kèm
+2. Chờ tải xong</t>
         </is>
       </c>
       <c r="H71" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tệp: bien-ban.pdf</t>
         </is>
       </c>
       <c r="I71" s="15" t="inlineStr">
         <is>
-          <t>- Lưu thành công, quay về danh sách
-- Phiếu mới ở trạng thái “Đang tạo”, đã có số phiếu
-- ⚠️ Lưu nháp KHÔNG đòi Nguyên nhân / Hành động</t>
+          <t>- Trong lúc tải có báo đang tải lên
+- Xong thì hiện biểu tượng loại tệp, tên tệp và 3 nút Tải xuống / Thay đổi / Xóa</t>
         </is>
       </c>
       <c r="J71" s="15" t="inlineStr"/>
@@ -4558,25 +4560,162 @@
       </c>
       <c r="C72" s="16" t="inlineStr">
         <is>
+          <t>TC_04.012</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>Chặn đính kèm tệp sai định dạng</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>Có sẵn tệp .txt.</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>1. Chọn tệp .txt ở cột File đính kèm</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>Tệp: ghi-chu.txt</t>
+        </is>
+      </c>
+      <c r="I72" s="15" t="inlineStr">
+        <is>
+          <t>- Báo chỉ nhận tệp PDF, ảnh, Word hoặc Excel
+- Không tệp nào được gắn vào dòng</t>
+        </is>
+      </c>
+      <c r="J72" s="15" t="inlineStr"/>
+      <c r="K72" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L72" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N72" s="15" t="inlineStr"/>
+      <c r="O72" s="16" t="inlineStr"/>
+      <c r="P72" s="16" t="inlineStr"/>
+      <c r="Q72" s="16" t="inlineStr"/>
+    </row>
+    <row r="73" ht="45" customHeight="1">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
+        </is>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>TC_04.013</t>
+        </is>
+      </c>
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>Lưu nháp</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>Đang ở màn lập phiếu, chưa chọn nguyên nhân và hành động.</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Lưu nháp</t>
+        </is>
+      </c>
+      <c r="H73" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I73" s="15" t="inlineStr">
+        <is>
+          <t>- Lưu thành công, quay về danh sách
+- Phiếu mới ở trạng thái “Đang tạo”, đã có số phiếu
+- ⚠️ Lưu nháp KHÔNG đòi Nguyên nhân / Hành động</t>
+        </is>
+      </c>
+      <c r="J73" s="15" t="inlineStr"/>
+      <c r="K73" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L73" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N73" s="15" t="inlineStr"/>
+      <c r="O73" s="16" t="inlineStr"/>
+      <c r="P73" s="16" t="inlineStr"/>
+      <c r="Q73" s="16" t="inlineStr"/>
+    </row>
+    <row r="74" ht="34" customHeight="1">
+      <c r="A74" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
+        </is>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
           <t>TC_04.014</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="D74" s="15" t="inlineStr">
         <is>
           <t>Sửa phiếu nháp</t>
         </is>
       </c>
-      <c r="E72" s="16" t="inlineStr">
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F72" s="15" t="inlineStr">
+      <c r="F74" s="15" t="inlineStr">
         <is>
           <t>Phiếu nháp do chính người đăng nhập lập.</t>
         </is>
       </c>
-      <c r="G72" s="15" t="inlineStr">
+      <c r="G74" s="15" t="inlineStr">
         <is>
           <t>1. Bấm Sửa ở dòng phiếu
 2. Chọn nguyên nhân và hành động
@@ -4584,152 +4723,15 @@
 4. Mở lại phiếu</t>
         </is>
       </c>
-      <c r="H72" s="15" t="inlineStr">
+      <c r="H74" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I72" s="15" t="inlineStr">
+      <c r="I74" s="15" t="inlineStr">
         <is>
           <t>- Lưu thành công, mở lại thấy đúng nguyên nhân + hành động đã chọn
 - Số phiếu KHÔNG đổi</t>
-        </is>
-      </c>
-      <c r="J72" s="15" t="inlineStr"/>
-      <c r="K72" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L72" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M72" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N72" s="15" t="inlineStr"/>
-      <c r="O72" s="16" t="inlineStr"/>
-      <c r="P72" s="16" t="inlineStr"/>
-      <c r="Q72" s="16" t="inlineStr"/>
-    </row>
-    <row r="73" ht="34" customHeight="1">
-      <c r="A73" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B73" s="15" t="inlineStr">
-        <is>
-          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
-        </is>
-      </c>
-      <c r="C73" s="16" t="inlineStr">
-        <is>
-          <t>TC_04.015</t>
-        </is>
-      </c>
-      <c r="D73" s="15" t="inlineStr">
-        <is>
-          <t>Xóa dòng thiết bị khỏi phiếu</t>
-        </is>
-      </c>
-      <c r="E73" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F73" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu đang sửa có 2 dòng thiết bị.</t>
-        </is>
-      </c>
-      <c r="G73" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm nút xóa ở dòng thứ 2
-2. Lưu nháp rồi mở lại phiếu</t>
-        </is>
-      </c>
-      <c r="H73" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I73" s="15" t="inlineStr">
-        <is>
-          <t>- Sau khi lưu, phiếu chỉ còn 1 dòng thiết bị</t>
-        </is>
-      </c>
-      <c r="J73" s="15" t="inlineStr"/>
-      <c r="K73" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L73" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M73" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N73" s="15" t="inlineStr"/>
-      <c r="O73" s="16" t="inlineStr"/>
-      <c r="P73" s="16" t="inlineStr"/>
-      <c r="Q73" s="16" t="inlineStr"/>
-    </row>
-    <row r="74" ht="34" customHeight="1">
-      <c r="A74" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B74" s="15" t="inlineStr">
-        <is>
-          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
-        </is>
-      </c>
-      <c r="C74" s="16" t="inlineStr">
-        <is>
-          <t>TC_04.016</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
-        <is>
-          <t>Cảnh báo khi thoát lúc chưa lưu</t>
-        </is>
-      </c>
-      <c r="E74" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F74" s="15" t="inlineStr">
-        <is>
-          <t>Đang ở màn lập phiếu.</t>
-        </is>
-      </c>
-      <c r="G74" s="15" t="inlineStr">
-        <is>
-          <t>1. Chọn một nguyên nhân
-2. Bấm Quay lại</t>
-        </is>
-      </c>
-      <c r="H74" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I74" s="15" t="inlineStr">
-        <is>
-          <t>- Hiện cửa sổ “Thông tin chưa lưu”
-- Bấm Ở lại thì dữ liệu còn nguyên; bấm Thoát mới rời đi</t>
         </is>
       </c>
       <c r="J74" s="15" t="inlineStr"/>
@@ -4766,28 +4768,28 @@
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>TC_04.017</t>
+          <t>TC_04.015</t>
         </is>
       </c>
       <c r="D75" s="15" t="inlineStr">
         <is>
-          <t>Bảng thiết bị cuộn ngang được ở cả trên và dưới</t>
+          <t>Xóa dòng thiết bị khỏi phiếu</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F75" s="15" t="inlineStr">
         <is>
-          <t>Thu hẹp cửa sổ trình duyệt để bảng bị tràn ngang.</t>
+          <t>Phiếu đang sửa có 2 dòng thiết bị.</t>
         </is>
       </c>
       <c r="G75" s="15" t="inlineStr">
         <is>
-          <t>1. Kéo thanh cuộn phía TRÊN bảng
-2. Kéo thanh cuộn phía DƯỚI bảng</t>
+          <t>1. Bấm nút xóa ở dòng thứ 2
+2. Lưu nháp rồi mở lại phiếu</t>
         </is>
       </c>
       <c r="H75" s="15" t="inlineStr">
@@ -4797,8 +4799,7 @@
       </c>
       <c r="I75" s="15" t="inlineStr">
         <is>
-          <t>- Có thanh cuộn ở cả trên và dưới, kéo bên nào bên kia chạy theo
-- Phóng rộng thì thanh trên tự ẩn</t>
+          <t>- Sau khi lưu, phiếu chỉ còn 1 dòng thiết bị</t>
         </is>
       </c>
       <c r="J75" s="15" t="inlineStr"/>
@@ -4822,30 +4823,76 @@
       <c r="P75" s="16" t="inlineStr"/>
       <c r="Q75" s="16" t="inlineStr"/>
     </row>
-    <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="13" t="n"/>
-      <c r="B76" s="13" t="n"/>
-      <c r="C76" s="14" t="inlineStr">
-        <is>
-          <t>V. GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="n"/>
-      <c r="E76" s="4" t="n"/>
-      <c r="F76" s="4" t="n"/>
-      <c r="G76" s="4" t="n"/>
-      <c r="H76" s="4" t="n"/>
-      <c r="I76" s="4" t="n"/>
-      <c r="J76" s="4" t="n"/>
-      <c r="K76" s="4" t="n"/>
-      <c r="L76" s="4" t="n"/>
-      <c r="M76" s="4" t="n"/>
-      <c r="N76" s="4" t="n"/>
-      <c r="O76" s="4" t="n"/>
-      <c r="P76" s="4" t="n"/>
-      <c r="Q76" s="5" t="n"/>
-    </row>
-    <row r="77" ht="43" customHeight="1">
+    <row r="76" ht="34" customHeight="1">
+      <c r="A76" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B76" s="15" t="inlineStr">
+        <is>
+          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>TC_04.016</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="inlineStr">
+        <is>
+          <t>Cảnh báo khi thoát lúc chưa lưu</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Đang ở màn lập phiếu.</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="inlineStr">
+        <is>
+          <t>1. Chọn một nguyên nhân
+2. Bấm Quay lại</t>
+        </is>
+      </c>
+      <c r="H76" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I76" s="15" t="inlineStr">
+        <is>
+          <t>- Hiện cửa sổ “Thông tin chưa lưu”
+- Bấm Ở lại thì dữ liệu còn nguyên; bấm Thoát mới rời đi</t>
+        </is>
+      </c>
+      <c r="J76" s="15" t="inlineStr"/>
+      <c r="K76" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L76" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N76" s="15" t="inlineStr"/>
+      <c r="O76" s="16" t="inlineStr"/>
+      <c r="P76" s="16" t="inlineStr"/>
+      <c r="Q76" s="16" t="inlineStr"/>
+    </row>
+    <row r="77" ht="34" customHeight="1">
       <c r="A77" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -4853,33 +4900,33 @@
       </c>
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+          <t>LẬP PHIẾU, SỬA &amp; XEM</t>
         </is>
       </c>
       <c r="C77" s="16" t="inlineStr">
         <is>
-          <t>TC_05.001</t>
+          <t>TC_04.017</t>
         </is>
       </c>
       <c r="D77" s="15" t="inlineStr">
         <is>
-          <t>Gửi phiếu đi để cung cấp thông tin</t>
+          <t>Bảng thiết bị cuộn ngang được ở cả trên và dưới</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F77" s="15" t="inlineStr">
         <is>
-          <t>Phiếu nháp có 1 thiết bị, đã chọn nguyên nhân và hành động “Cung cấp thông tin làm báo giá”.</t>
+          <t>Thu hẹp cửa sổ trình duyệt để bảng bị tràn ngang.</t>
         </is>
       </c>
       <c r="G77" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm “Lưu và gửi”
-2. Xác nhận ở cửa sổ hỏi lại</t>
+          <t>1. Kéo thanh cuộn phía TRÊN bảng
+2. Kéo thanh cuộn phía DƯỚI bảng</t>
         </is>
       </c>
       <c r="H77" s="15" t="inlineStr">
@@ -4889,9 +4936,8 @@
       </c>
       <c r="I77" s="15" t="inlineStr">
         <is>
-          <t>- Phiếu chuyển sang “Chờ CCTT”
-- Ghi nhận thời điểm gửi
-- Phiếu yêu cầu GỐC chuyển sang “Đã xử lý”, điền Người xử lý và Ngày xử lý</t>
+          <t>- Có thanh cuộn ở cả trên và dưới, kéo bên nào bên kia chạy theo
+- Phóng rộng thì thanh trên tự ẩn</t>
         </is>
       </c>
       <c r="J77" s="15" t="inlineStr"/>
@@ -4915,49 +4961,142 @@
       <c r="P77" s="16" t="inlineStr"/>
       <c r="Q77" s="16" t="inlineStr"/>
     </row>
-    <row r="78" ht="74" customHeight="1">
-      <c r="A78" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B78" s="15" t="inlineStr">
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="13" t="n"/>
+      <c r="B78" s="13" t="n"/>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>V. GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="n"/>
+      <c r="E78" s="4" t="n"/>
+      <c r="F78" s="4" t="n"/>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="n"/>
+      <c r="J78" s="4" t="n"/>
+      <c r="K78" s="4" t="n"/>
+      <c r="L78" s="4" t="n"/>
+      <c r="M78" s="4" t="n"/>
+      <c r="N78" s="4" t="n"/>
+      <c r="O78" s="4" t="n"/>
+      <c r="P78" s="4" t="n"/>
+      <c r="Q78" s="5" t="n"/>
+    </row>
+    <row r="79" ht="43" customHeight="1">
+      <c r="A79" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
         </is>
       </c>
-      <c r="C78" s="16" t="inlineStr">
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>TC_05.001</t>
+        </is>
+      </c>
+      <c r="D79" s="15" t="inlineStr">
+        <is>
+          <t>Gửi phiếu đi để cung cấp thông tin</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F79" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu nháp có 1 thiết bị, đã chọn nguyên nhân và hành động “Cung cấp thông tin làm báo giá”.</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm “Lưu và gửi”
+2. Xác nhận ở cửa sổ hỏi lại</t>
+        </is>
+      </c>
+      <c r="H79" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="15" t="inlineStr">
+        <is>
+          <t>- Phiếu chuyển sang “Chờ CCTT”
+- Ghi nhận thời điểm gửi
+- Phiếu yêu cầu GỐC chuyển sang “Đã xử lý”, điền Người xử lý và Ngày xử lý</t>
+        </is>
+      </c>
+      <c r="J79" s="15" t="inlineStr"/>
+      <c r="K79" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L79" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M79" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N79" s="15" t="inlineStr"/>
+      <c r="O79" s="16" t="inlineStr"/>
+      <c r="P79" s="16" t="inlineStr"/>
+      <c r="Q79" s="16" t="inlineStr"/>
+    </row>
+    <row r="80" ht="74" customHeight="1">
+      <c r="A80" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>TC_05.002</t>
         </is>
       </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="D80" s="15" t="inlineStr">
         <is>
           <t>Thông báo cho người lập phiếu cung cấp thông tin</t>
         </is>
       </c>
-      <c r="E78" s="16" t="inlineStr">
+      <c r="E80" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F78" s="15" t="inlineStr">
+      <c r="F80" s="15" t="inlineStr">
         <is>
           <t>Công ty có 7 người được cấp quyền “Tạo phiếu cung cấp thông tin”.</t>
         </is>
       </c>
-      <c r="G78" s="15" t="inlineStr">
+      <c r="G80" s="15" t="inlineStr">
         <is>
           <t>1. Gửi phiếu đi
 2. Đăng nhập lần lượt bằng vài người trong số đó, mở chuông thông báo</t>
         </is>
       </c>
-      <c r="H78" s="15" t="inlineStr">
+      <c r="H80" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I78" s="15" t="inlineStr">
+      <c r="I80" s="15" t="inlineStr">
         <is>
           <t>- Những người có quyền đó và CÙNG CÔNG TY đều nhận được thông báo
 - Nội dung dạng: [PXL] Chờ duyệt: &lt;số phiếu&gt;. Khách hàng: &lt;tên khách&gt;.
@@ -4965,144 +5104,6 @@
 - ⚠️ Thông báo đi theo QUYỀN, không theo phòng ban</t>
         </is>
       </c>
-      <c r="J78" s="15" t="inlineStr"/>
-      <c r="K78" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L78" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M78" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N78" s="15" t="inlineStr"/>
-      <c r="O78" s="16" t="inlineStr"/>
-      <c r="P78" s="16" t="inlineStr"/>
-      <c r="Q78" s="16" t="inlineStr"/>
-    </row>
-    <row r="79" ht="72" customHeight="1">
-      <c r="A79" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B79" s="15" t="inlineStr">
-        <is>
-          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
-        </is>
-      </c>
-      <c r="C79" s="16" t="inlineStr">
-        <is>
-          <t>TC_05.003</t>
-        </is>
-      </c>
-      <c r="D79" s="15" t="inlineStr">
-        <is>
-          <t>Mọi thiết bị đều Tư vấn điện thoại</t>
-        </is>
-      </c>
-      <c r="E79" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F79" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu có 1 thiết bị duy nhất, chọn hành động “Tư vấn điện thoại” và đã nhập nội dung xử lý.</t>
-        </is>
-      </c>
-      <c r="G79" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm nút “Lưu nháp” (KHÔNG bấm Lưu và gửi)
-2. Xem trạng thái phiếu và phiếu yêu cầu gốc</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="inlineStr">
-        <is>
-          <t>Nội dung xử lý: “Đã hướng dẫn khách kiểm tra nguồn điện”</t>
-        </is>
-      </c>
-      <c r="I79" s="15" t="inlineStr">
-        <is>
-          <t>- ⚠️ Phiếu vẫn chuyển thành “Đã tư vấn điện thoại” dù bấm Lưu nháp — đây là hành vi đúng
-- Phiếu yêu cầu gốc cũng chuyển “Đã tư vấn điện thoại”, luồng kết thúc tại đây
-- Không ai nhận thông báo chờ cung cấp thông tin</t>
-        </is>
-      </c>
-      <c r="J79" s="15" t="inlineStr"/>
-      <c r="K79" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L79" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M79" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N79" s="15" t="inlineStr"/>
-      <c r="O79" s="16" t="inlineStr"/>
-      <c r="P79" s="16" t="inlineStr"/>
-      <c r="Q79" s="16" t="inlineStr"/>
-    </row>
-    <row r="80" ht="38" customHeight="1">
-      <c r="A80" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B80" s="15" t="inlineStr">
-        <is>
-          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
-        </is>
-      </c>
-      <c r="C80" s="16" t="inlineStr">
-        <is>
-          <t>TC_05.004</t>
-        </is>
-      </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu nhiều thiết bị, chỉ một dòng cần báo giá</t>
-        </is>
-      </c>
-      <c r="E80" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F80" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu có 2 thiết bị: dòng 1 chọn Tư vấn điện thoại (có nội dung xử lý), dòng 2 chọn Cung cấp thông tin làm báo giá.</t>
-        </is>
-      </c>
-      <c r="G80" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm Lưu và gửi, xác nhận</t>
-        </is>
-      </c>
-      <c r="H80" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I80" s="15" t="inlineStr">
-        <is>
-          <t>- Phiếu chuyển sang “Chờ CCTT” (KHÔNG phải Đã tư vấn điện thoại)
-- Phiếu yêu cầu gốc chuyển “Đã xử lý”</t>
-        </is>
-      </c>
       <c r="J80" s="15" t="inlineStr"/>
       <c r="K80" s="16" t="inlineStr">
         <is>
@@ -5124,7 +5125,7 @@
       <c r="P80" s="16" t="inlineStr"/>
       <c r="Q80" s="16" t="inlineStr"/>
     </row>
-    <row r="81" ht="57" customHeight="1">
+    <row r="81" ht="72" customHeight="1">
       <c r="A81" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -5137,25 +5138,163 @@
       </c>
       <c r="C81" s="16" t="inlineStr">
         <is>
+          <t>TC_05.003</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Mọi thiết bị đều Tư vấn điện thoại</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu có 1 thiết bị duy nhất, chọn hành động “Tư vấn điện thoại” và đã nhập nội dung xử lý.</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm nút “Lưu nháp” (KHÔNG bấm Lưu và gửi)
+2. Xem trạng thái phiếu và phiếu yêu cầu gốc</t>
+        </is>
+      </c>
+      <c r="H81" s="15" t="inlineStr">
+        <is>
+          <t>Nội dung xử lý: “Đã hướng dẫn khách kiểm tra nguồn điện”</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>- ⚠️ Phiếu vẫn chuyển thành “Đã tư vấn điện thoại” dù bấm Lưu nháp — đây là hành vi đúng
+- Phiếu yêu cầu gốc cũng chuyển “Đã tư vấn điện thoại”, luồng kết thúc tại đây
+- Không ai nhận thông báo chờ cung cấp thông tin</t>
+        </is>
+      </c>
+      <c r="J81" s="15" t="inlineStr"/>
+      <c r="K81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N81" s="15" t="inlineStr"/>
+      <c r="O81" s="16" t="inlineStr"/>
+      <c r="P81" s="16" t="inlineStr"/>
+      <c r="Q81" s="16" t="inlineStr"/>
+    </row>
+    <row r="82" ht="38" customHeight="1">
+      <c r="A82" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>TC_05.004</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu nhiều thiết bị, chỉ một dòng cần báo giá</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu có 2 thiết bị: dòng 1 chọn Tư vấn điện thoại (có nội dung xử lý), dòng 2 chọn Cung cấp thông tin làm báo giá.</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Lưu và gửi, xác nhận</t>
+        </is>
+      </c>
+      <c r="H82" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="15" t="inlineStr">
+        <is>
+          <t>- Phiếu chuyển sang “Chờ CCTT” (KHÔNG phải Đã tư vấn điện thoại)
+- Phiếu yêu cầu gốc chuyển “Đã xử lý”</t>
+        </is>
+      </c>
+      <c r="J82" s="15" t="inlineStr"/>
+      <c r="K82" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L82" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M82" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N82" s="15" t="inlineStr"/>
+      <c r="O82" s="16" t="inlineStr"/>
+      <c r="P82" s="16" t="inlineStr"/>
+      <c r="Q82" s="16" t="inlineStr"/>
+    </row>
+    <row r="83" ht="57" customHeight="1">
+      <c r="A83" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+        </is>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
           <t>TC_05.005</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="D83" s="15" t="inlineStr">
         <is>
           <t>Không duyệt phiếu</t>
         </is>
       </c>
-      <c r="E81" s="16" t="inlineStr">
+      <c r="E83" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F81" s="15" t="inlineStr">
+      <c r="F83" s="15" t="inlineStr">
         <is>
           <t>Phiếu đang “Chờ CCTT”, người đăng nhập có quyền “Tạo phiếu cung cấp thông tin”. Phiếu do nhân viên G lập.</t>
         </is>
       </c>
-      <c r="G81" s="15" t="inlineStr">
+      <c r="G83" s="15" t="inlineStr">
         <is>
           <t>1. Bấm “Không duyệt” ở dòng phiếu
 2. Nhập lý do
@@ -5163,153 +5302,16 @@
 4. Đăng nhập bằng G, mở chuông thông báo và mở phiếu</t>
         </is>
       </c>
-      <c r="H81" s="15" t="inlineStr">
+      <c r="H83" s="15" t="inlineStr">
         <is>
           <t>Lý do: “Thiếu thông tin báo giá”</t>
         </is>
       </c>
-      <c r="I81" s="15" t="inlineStr">
+      <c r="I83" s="15" t="inlineStr">
         <is>
           <t>- Phiếu trở lại “Đang tạo”, lý do lưu trên phiếu và hiện ở khối thông tin (chữ xám)
 - G nhận thông báo: [PXL] Từ chối: &lt;số phiếu&gt;. Lý do: …
 - G sửa lại và gửi lần nữa được</t>
-        </is>
-      </c>
-      <c r="J81" s="15" t="inlineStr"/>
-      <c r="K81" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L81" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M81" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N81" s="15" t="inlineStr"/>
-      <c r="O81" s="16" t="inlineStr"/>
-      <c r="P81" s="16" t="inlineStr"/>
-      <c r="Q81" s="16" t="inlineStr"/>
-    </row>
-    <row r="82" ht="34" customHeight="1">
-      <c r="A82" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B82" s="15" t="inlineStr">
-        <is>
-          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
-        </is>
-      </c>
-      <c r="C82" s="16" t="inlineStr">
-        <is>
-          <t>TC_05.006</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>Không duyệt mà bỏ trống lý do</t>
-        </is>
-      </c>
-      <c r="E82" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F82" s="15" t="inlineStr">
-        <is>
-          <t>Popup Không duyệt đang mở.</t>
-        </is>
-      </c>
-      <c r="G82" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm nút Không duyệt</t>
-        </is>
-      </c>
-      <c r="H82" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I82" s="15" t="inlineStr">
-        <is>
-          <t>- Báo lỗi đỏ dưới ô Lý do không duyệt
-- Popup không đóng, phiếu chưa đổi trạng thái</t>
-        </is>
-      </c>
-      <c r="J82" s="15" t="inlineStr"/>
-      <c r="K82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M82" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N82" s="15" t="inlineStr"/>
-      <c r="O82" s="16" t="inlineStr"/>
-      <c r="P82" s="16" t="inlineStr"/>
-      <c r="Q82" s="16" t="inlineStr"/>
-    </row>
-    <row r="83" ht="49" customHeight="1">
-      <c r="A83" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
-        </is>
-      </c>
-      <c r="C83" s="16" t="inlineStr">
-        <is>
-          <t>TC_05.007</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>Không duyệt KHÔNG trả phiếu yêu cầu gốc về Chờ xử lý</t>
-        </is>
-      </c>
-      <c r="E83" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F83" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý đang “Chờ CCTT”, phiếu yêu cầu gốc đang “Đã xử lý”.</t>
-        </is>
-      </c>
-      <c r="G83" s="15" t="inlineStr">
-        <is>
-          <t>1. Không duyệt phiếu xử lý
-2. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành, tìm phiếu gốc</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="inlineStr">
-        <is>
-          <t>Lý do: “test”</t>
-        </is>
-      </c>
-      <c r="I83" s="15" t="inlineStr">
-        <is>
-          <t>- Phiếu xử lý về “Đang tạo”
-- ⚠️ Phiếu yêu cầu gốc VẪN là “Đã xử lý”, không quay lại “Chờ xử lý” — đúng nghiệp vụ, chỉ khi XÓA phiếu xử lý mới trả về</t>
         </is>
       </c>
       <c r="J83" s="15" t="inlineStr"/>
@@ -5346,37 +5348,38 @@
       </c>
       <c r="C84" s="16" t="inlineStr">
         <is>
-          <t>TC_05.008</t>
+          <t>TC_05.006</t>
         </is>
       </c>
       <c r="D84" s="15" t="inlineStr">
         <is>
-          <t>Không duyệt lần 2 khi phiếu đã về Đang tạo</t>
+          <t>Không duyệt mà bỏ trống lý do</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F84" s="15" t="inlineStr">
         <is>
-          <t>Phiếu vừa bị Không duyệt, đang ở “Đang tạo”.</t>
+          <t>Popup Không duyệt đang mở.</t>
         </is>
       </c>
       <c r="G84" s="15" t="inlineStr">
         <is>
-          <t>1. Dùng công cụ kiểm thử API gọi lại chức năng Không duyệt</t>
+          <t>1. Bấm nút Không duyệt</t>
         </is>
       </c>
       <c r="H84" s="15" t="inlineStr">
         <is>
-          <t>Lý do: “lần 2”</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I84" s="15" t="inlineStr">
         <is>
-          <t>- Hệ thống chặn, báo phiếu không ở trạng thái Chờ CCTT</t>
+          <t>- Báo lỗi đỏ dưới ô Lý do không duyệt
+- Popup không đóng, phiếu chưa đổi trạng thái</t>
         </is>
       </c>
       <c r="J84" s="15" t="inlineStr"/>
@@ -5400,7 +5403,7 @@
       <c r="P84" s="16" t="inlineStr"/>
       <c r="Q84" s="16" t="inlineStr"/>
     </row>
-    <row r="85" ht="56" customHeight="1">
+    <row r="85" ht="49" customHeight="1">
       <c r="A85" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -5413,38 +5416,39 @@
       </c>
       <c r="C85" s="16" t="inlineStr">
         <is>
-          <t>TC_05.009</t>
+          <t>TC_05.007</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
         <is>
-          <t>Tạo phiếu cung cấp thông tin</t>
+          <t>Không duyệt KHÔNG trả phiếu yêu cầu gốc về Chờ xử lý</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F85" s="15" t="inlineStr">
         <is>
-          <t>Phiếu đang “Chờ CCTT”, người đăng nhập có quyền tương ứng.</t>
+          <t>Phiếu xử lý đang “Chờ CCTT”, phiếu yêu cầu gốc đang “Đã xử lý”.</t>
         </is>
       </c>
       <c r="G85" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm “Tạo phiếu cung cấp thông tin”</t>
+          <t>1. Không duyệt phiếu xử lý
+2. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành, tìm phiếu gốc</t>
         </is>
       </c>
       <c r="H85" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Lý do: “test”</t>
         </is>
       </c>
       <c r="I85" s="15" t="inlineStr">
         <is>
-          <t>- ⚠️ Màn Phiếu cung cấp thông tin chưa có trên hệ thống mới: hệ thống báo hướng dẫn xử lý tạm trên phần mềm ERP
-- Khi màn đó hoàn thành sẽ chuyển thẳng sang màn lập phiếu</t>
+          <t>- Phiếu xử lý về “Đang tạo”
+- ⚠️ Phiếu yêu cầu gốc VẪN là “Đã xử lý”, không quay lại “Chờ xử lý” — đúng nghiệp vụ, chỉ khi XÓA phiếu xử lý mới trả về</t>
         </is>
       </c>
       <c r="J85" s="15" t="inlineStr"/>
@@ -5468,30 +5472,74 @@
       <c r="P85" s="16" t="inlineStr"/>
       <c r="Q85" s="16" t="inlineStr"/>
     </row>
-    <row r="86" ht="26" customHeight="1">
-      <c r="A86" s="13" t="n"/>
-      <c r="B86" s="13" t="n"/>
-      <c r="C86" s="14" t="inlineStr">
-        <is>
-          <t>VI. XÓA</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="n"/>
-      <c r="E86" s="4" t="n"/>
-      <c r="F86" s="4" t="n"/>
-      <c r="G86" s="4" t="n"/>
-      <c r="H86" s="4" t="n"/>
-      <c r="I86" s="4" t="n"/>
-      <c r="J86" s="4" t="n"/>
-      <c r="K86" s="4" t="n"/>
-      <c r="L86" s="4" t="n"/>
-      <c r="M86" s="4" t="n"/>
-      <c r="N86" s="4" t="n"/>
-      <c r="O86" s="4" t="n"/>
-      <c r="P86" s="4" t="n"/>
-      <c r="Q86" s="5" t="n"/>
-    </row>
-    <row r="87" ht="69" customHeight="1">
+    <row r="86" ht="34" customHeight="1">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="inlineStr">
+        <is>
+          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>TC_05.008</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="inlineStr">
+        <is>
+          <t>Không duyệt lần 2 khi phiếu đã về Đang tạo</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F86" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu vừa bị Không duyệt, đang ở “Đang tạo”.</t>
+        </is>
+      </c>
+      <c r="G86" s="15" t="inlineStr">
+        <is>
+          <t>1. Dùng công cụ kiểm thử API gọi lại chức năng Không duyệt</t>
+        </is>
+      </c>
+      <c r="H86" s="15" t="inlineStr">
+        <is>
+          <t>Lý do: “lần 2”</t>
+        </is>
+      </c>
+      <c r="I86" s="15" t="inlineStr">
+        <is>
+          <t>- Hệ thống chặn, báo phiếu không ở trạng thái Chờ CCTT</t>
+        </is>
+      </c>
+      <c r="J86" s="15" t="inlineStr"/>
+      <c r="K86" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L86" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M86" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N86" s="15" t="inlineStr"/>
+      <c r="O86" s="16" t="inlineStr"/>
+      <c r="P86" s="16" t="inlineStr"/>
+      <c r="Q86" s="16" t="inlineStr"/>
+    </row>
+    <row r="87" ht="56" customHeight="1">
       <c r="A87" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -5499,34 +5547,32 @@
       </c>
       <c r="B87" s="15" t="inlineStr">
         <is>
-          <t>XÓA</t>
+          <t>GỬI DUYỆT &amp; KHÔNG DUYỆT</t>
         </is>
       </c>
       <c r="C87" s="16" t="inlineStr">
         <is>
-          <t>TC_06.001</t>
+          <t>TC_05.009</t>
         </is>
       </c>
       <c r="D87" s="15" t="inlineStr">
         <is>
-          <t>Xóa phiếu nháp và trả phiếu yêu cầu về Chờ xử lý</t>
+          <t>Tạo phiếu cung cấp thông tin</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F87" s="15" t="inlineStr">
         <is>
-          <t>Phiếu xử lý “Đang tạo” do chính người đăng nhập lập; phiếu yêu cầu gốc đang “Đã xử lý”.</t>
+          <t>Phiếu đang “Chờ CCTT”, người đăng nhập có quyền tương ứng.</t>
         </is>
       </c>
       <c r="G87" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Xóa ở dòng phiếu
-2. Xác nhận
-3. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành, tìm phiếu yêu cầu gốc</t>
+          <t>1. Bấm “Tạo phiếu cung cấp thông tin”</t>
         </is>
       </c>
       <c r="H87" s="15" t="inlineStr">
@@ -5536,9 +5582,8 @@
       </c>
       <c r="I87" s="15" t="inlineStr">
         <is>
-          <t>- Cửa sổ hỏi “Bạn có chắc muốn xóa phiếu '&lt;số phiếu&gt;'?”
-- Phiếu xử lý biến mất khỏi danh sách
-- ⚠️ Phiếu yêu cầu gốc TRỞ LẠI “Chờ xử lý”, xóa Người xử lý và Ngày xử lý, và lại có nút “Tạo phiếu xử lý yêu cầu”</t>
+          <t>- ⚠️ Màn Phiếu cung cấp thông tin chưa có trên hệ thống mới: hệ thống báo hướng dẫn xử lý tạm trên phần mềm ERP
+- Khi màn đó hoàn thành sẽ chuyển thẳng sang màn lập phiếu</t>
         </is>
       </c>
       <c r="J87" s="15" t="inlineStr"/>
@@ -5562,118 +5607,77 @@
       <c r="P87" s="16" t="inlineStr"/>
       <c r="Q87" s="16" t="inlineStr"/>
     </row>
-    <row r="88" ht="34" customHeight="1">
-      <c r="A88" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B88" s="15" t="inlineStr">
+    <row r="88" ht="26" customHeight="1">
+      <c r="A88" s="13" t="n"/>
+      <c r="B88" s="13" t="n"/>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>VI. XÓA</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="n"/>
+      <c r="E88" s="4" t="n"/>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
+      <c r="L88" s="4" t="n"/>
+      <c r="M88" s="4" t="n"/>
+      <c r="N88" s="4" t="n"/>
+      <c r="O88" s="4" t="n"/>
+      <c r="P88" s="4" t="n"/>
+      <c r="Q88" s="5" t="n"/>
+    </row>
+    <row r="89" ht="69" customHeight="1">
+      <c r="A89" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
         <is>
           <t>XÓA</t>
         </is>
       </c>
-      <c r="C88" s="16" t="inlineStr">
-        <is>
-          <t>TC_06.002</t>
-        </is>
-      </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>Hủy ở cửa sổ xác nhận xóa</t>
-        </is>
-      </c>
-      <c r="E88" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F88" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu nháp của chính mình.</t>
-        </is>
-      </c>
-      <c r="G88" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm Xóa
-2. Bấm Hủy</t>
-        </is>
-      </c>
-      <c r="H88" s="15" t="inlineStr">
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>TC_06.001</t>
+        </is>
+      </c>
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>Xóa phiếu nháp và trả phiếu yêu cầu về Chờ xử lý</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F89" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý “Đang tạo” do chính người đăng nhập lập; phiếu yêu cầu gốc đang “Đã xử lý”.</t>
+        </is>
+      </c>
+      <c r="G89" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Xóa ở dòng phiếu
+2. Xác nhận
+3. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành, tìm phiếu yêu cầu gốc</t>
+        </is>
+      </c>
+      <c r="H89" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I88" s="15" t="inlineStr">
-        <is>
-          <t>- Phiếu vẫn còn nguyên, phiếu yêu cầu gốc không đổi</t>
-        </is>
-      </c>
-      <c r="J88" s="15" t="inlineStr"/>
-      <c r="K88" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L88" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M88" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N88" s="15" t="inlineStr"/>
-      <c r="O88" s="16" t="inlineStr"/>
-      <c r="P88" s="16" t="inlineStr"/>
-      <c r="Q88" s="16" t="inlineStr"/>
-    </row>
-    <row r="89" ht="34" customHeight="1">
-      <c r="A89" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B89" s="15" t="inlineStr">
-        <is>
-          <t>XÓA</t>
-        </is>
-      </c>
-      <c r="C89" s="16" t="inlineStr">
-        <is>
-          <t>TC_06.003</t>
-        </is>
-      </c>
-      <c r="D89" s="15" t="inlineStr">
-        <is>
-          <t>Không có nút Xóa với phiếu đã gửi</t>
-        </is>
-      </c>
-      <c r="E89" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F89" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu đang “Chờ CCTT” do chính mình lập.</t>
-        </is>
-      </c>
-      <c r="G89" s="15" t="inlineStr">
-        <is>
-          <t>1. Xem cột Hành động ở danh sách và ở màn chi tiết</t>
-        </is>
-      </c>
-      <c r="H89" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I89" s="15" t="inlineStr">
         <is>
-          <t>- Không có nút Sửa và Xóa ở cả hai nơi</t>
+          <t>- Cửa sổ hỏi “Bạn có chắc muốn xóa phiếu '&lt;số phiếu&gt;'?”
+- Phiếu xử lý biến mất khỏi danh sách
+- ⚠️ Phiếu yêu cầu gốc TRỞ LẠI “Chờ xử lý”, xóa Người xử lý và Ngày xử lý, và lại có nút “Tạo phiếu xử lý yêu cầu”</t>
         </is>
       </c>
       <c r="J89" s="15" t="inlineStr"/>
@@ -5697,28 +5701,73 @@
       <c r="P89" s="16" t="inlineStr"/>
       <c r="Q89" s="16" t="inlineStr"/>
     </row>
-    <row r="90" ht="26" customHeight="1">
-      <c r="A90" s="13" t="n"/>
-      <c r="B90" s="13" t="n"/>
-      <c r="C90" s="14" t="inlineStr">
-        <is>
-          <t>VII. XUẤT EXCEL / IN</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="n"/>
-      <c r="E90" s="4" t="n"/>
-      <c r="F90" s="4" t="n"/>
-      <c r="G90" s="4" t="n"/>
-      <c r="H90" s="4" t="n"/>
-      <c r="I90" s="4" t="n"/>
-      <c r="J90" s="4" t="n"/>
-      <c r="K90" s="4" t="n"/>
-      <c r="L90" s="4" t="n"/>
-      <c r="M90" s="4" t="n"/>
-      <c r="N90" s="4" t="n"/>
-      <c r="O90" s="4" t="n"/>
-      <c r="P90" s="4" t="n"/>
-      <c r="Q90" s="5" t="n"/>
+    <row r="90" ht="34" customHeight="1">
+      <c r="A90" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>XÓA</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>TC_06.002</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>Hủy ở cửa sổ xác nhận xóa</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F90" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu nháp của chính mình.</t>
+        </is>
+      </c>
+      <c r="G90" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Xóa
+2. Bấm Hủy</t>
+        </is>
+      </c>
+      <c r="H90" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I90" s="15" t="inlineStr">
+        <is>
+          <t>- Phiếu vẫn còn nguyên, phiếu yêu cầu gốc không đổi</t>
+        </is>
+      </c>
+      <c r="J90" s="15" t="inlineStr"/>
+      <c r="K90" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L90" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M90" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N90" s="15" t="inlineStr"/>
+      <c r="O90" s="16" t="inlineStr"/>
+      <c r="P90" s="16" t="inlineStr"/>
+      <c r="Q90" s="16" t="inlineStr"/>
     </row>
     <row r="91" ht="34" customHeight="1">
       <c r="A91" s="15" t="inlineStr">
@@ -5728,17 +5777,17 @@
       </c>
       <c r="B91" s="15" t="inlineStr">
         <is>
-          <t>XUẤT EXCEL / IN</t>
+          <t>XÓA</t>
         </is>
       </c>
       <c r="C91" s="16" t="inlineStr">
         <is>
-          <t>TC_07.001</t>
+          <t>TC_06.003</t>
         </is>
       </c>
       <c r="D91" s="15" t="inlineStr">
         <is>
-          <t>Xuất Excel theo bộ lọc</t>
+          <t>Không có nút Xóa với phiếu đã gửi</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
@@ -5748,14 +5797,12 @@
       </c>
       <c r="F91" s="15" t="inlineStr">
         <is>
-          <t>Đang lọc trạng thái “Chờ CCTT”, còn 22 phiếu.</t>
+          <t>Phiếu đang “Chờ CCTT” do chính mình lập.</t>
         </is>
       </c>
       <c r="G91" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Xuất Excel
-2. Giữ nguyên trường mặc định, bấm Xuất file
-3. Mở tệp</t>
+          <t>1. Xem cột Hành động ở danh sách và ở màn chi tiết</t>
         </is>
       </c>
       <c r="H91" s="15" t="inlineStr">
@@ -5765,9 +5812,7 @@
       </c>
       <c r="I91" s="15" t="inlineStr">
         <is>
-          <t>- Tệp tải về tên gợi nhớ tới màn hình
-- Có đúng 22 dòng dữ liệu
-- Cột đầu là STT</t>
+          <t>- Không có nút Sửa và Xóa ở cả hai nơi</t>
         </is>
       </c>
       <c r="J91" s="15" t="inlineStr"/>
@@ -5791,123 +5836,77 @@
       <c r="P91" s="16" t="inlineStr"/>
       <c r="Q91" s="16" t="inlineStr"/>
     </row>
-    <row r="92" ht="34" customHeight="1">
-      <c r="A92" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B92" s="15" t="inlineStr">
+    <row r="92" ht="26" customHeight="1">
+      <c r="A92" s="13" t="n"/>
+      <c r="B92" s="13" t="n"/>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>VII. XUẤT EXCEL / IN</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="n"/>
+      <c r="E92" s="4" t="n"/>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n"/>
+      <c r="I92" s="4" t="n"/>
+      <c r="J92" s="4" t="n"/>
+      <c r="K92" s="4" t="n"/>
+      <c r="L92" s="4" t="n"/>
+      <c r="M92" s="4" t="n"/>
+      <c r="N92" s="4" t="n"/>
+      <c r="O92" s="4" t="n"/>
+      <c r="P92" s="4" t="n"/>
+      <c r="Q92" s="5" t="n"/>
+    </row>
+    <row r="93" ht="34" customHeight="1">
+      <c r="A93" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
         <is>
           <t>XUẤT EXCEL / IN</t>
         </is>
       </c>
-      <c r="C92" s="16" t="inlineStr">
-        <is>
-          <t>TC_07.002</t>
-        </is>
-      </c>
-      <c r="D92" s="15" t="inlineStr">
-        <is>
-          <t>Chọn trường và thứ tự cột khi xuất</t>
-        </is>
-      </c>
-      <c r="E92" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F92" s="15" t="inlineStr">
-        <is>
-          <t>Cửa sổ chọn trường đang mở.</t>
-        </is>
-      </c>
-      <c r="G92" s="15" t="inlineStr">
-        <is>
-          <t>1. Bỏ chọn hết
-2. Chọn theo thứ tự: Số phiếu xử lý, Số phiếu yêu cầu, Trạng thái
-3. Xuất file</t>
-        </is>
-      </c>
-      <c r="H92" s="15" t="inlineStr">
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>TC_07.001</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>Xuất Excel theo bộ lọc</t>
+        </is>
+      </c>
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F93" s="15" t="inlineStr">
+        <is>
+          <t>Đang lọc trạng thái “Chờ CCTT”, còn 22 phiếu.</t>
+        </is>
+      </c>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm Xuất Excel
+2. Giữ nguyên trường mặc định, bấm Xuất file
+3. Mở tệp</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I92" s="15" t="inlineStr">
-        <is>
-          <t>- Tệp chỉ có 3 cột (cộng STT), đúng thứ tự vừa chọn</t>
-        </is>
-      </c>
-      <c r="J92" s="15" t="inlineStr"/>
-      <c r="K92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M92" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N92" s="15" t="inlineStr"/>
-      <c r="O92" s="16" t="inlineStr"/>
-      <c r="P92" s="16" t="inlineStr"/>
-      <c r="Q92" s="16" t="inlineStr"/>
-    </row>
-    <row r="93" ht="83" customHeight="1">
-      <c r="A93" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B93" s="15" t="inlineStr">
-        <is>
-          <t>XUẤT EXCEL / IN</t>
-        </is>
-      </c>
-      <c r="C93" s="16" t="inlineStr">
-        <is>
-          <t>TC_07.003</t>
-        </is>
-      </c>
-      <c r="D93" s="15" t="inlineStr">
-        <is>
-          <t>In một phiếu</t>
-        </is>
-      </c>
-      <c r="E93" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F93" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu đã điền đủ nguyên nhân và hành động.</t>
-        </is>
-      </c>
-      <c r="G93" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm In ở dòng phiếu
-2. Xem trang xem trước</t>
-        </is>
-      </c>
-      <c r="H93" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I93" s="15" t="inlineStr">
         <is>
-          <t>- Mở tab mới, thấy khung tờ giấy dọc, nền quanh giấy màu trắng
-- Bảng chi tiết có đủ 9 cột, trong đó có Nguyên nhân và Hành động
-- Có số phiếu xử lý, số phiếu yêu cầu, người yêu cầu, ngày nhận yêu cầu
-- Không còn chỗ nào bỏ trống dạng ký hiệu chờ điền</t>
+          <t>- Tệp tải về tên gợi nhớ tới màn hình
+- Có đúng 22 dòng dữ liệu
+- Cột đầu là STT</t>
         </is>
       </c>
       <c r="J93" s="15" t="inlineStr"/>
@@ -5944,28 +5943,29 @@
       </c>
       <c r="C94" s="16" t="inlineStr">
         <is>
-          <t>TC_07.004</t>
+          <t>TC_07.002</t>
         </is>
       </c>
       <c r="D94" s="15" t="inlineStr">
         <is>
-          <t>In danh sách theo bộ lọc</t>
+          <t>Chọn trường và thứ tự cột khi xuất</t>
         </is>
       </c>
       <c r="E94" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F94" s="15" t="inlineStr">
         <is>
-          <t>Đang lọc trạng thái “Đã tư vấn điện thoại”.</t>
+          <t>Cửa sổ chọn trường đang mở.</t>
         </is>
       </c>
       <c r="G94" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm In danh sách
-2. Xem trang xem trước</t>
+          <t>1. Bỏ chọn hết
+2. Chọn theo thứ tự: Số phiếu xử lý, Số phiếu yêu cầu, Trạng thái
+3. Xuất file</t>
         </is>
       </c>
       <c r="H94" s="15" t="inlineStr">
@@ -5975,8 +5975,7 @@
       </c>
       <c r="I94" s="15" t="inlineStr">
         <is>
-          <t>- Mở tab mới với mẫu danh sách khổ ngang, có khung tờ giấy
-- Bảng chứa đúng các phiếu đang lọc</t>
+          <t>- Tệp chỉ có 3 cột (cộng STT), đúng thứ tự vừa chọn</t>
         </is>
       </c>
       <c r="J94" s="15" t="inlineStr"/>
@@ -6000,7 +5999,7 @@
       <c r="P94" s="16" t="inlineStr"/>
       <c r="Q94" s="16" t="inlineStr"/>
     </row>
-    <row r="95" ht="42" customHeight="1">
+    <row r="95" ht="109" customHeight="1">
       <c r="A95" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -6013,28 +6012,28 @@
       </c>
       <c r="C95" s="16" t="inlineStr">
         <is>
-          <t>TC_07.005</t>
+          <t>TC_07.003</t>
         </is>
       </c>
       <c r="D95" s="15" t="inlineStr">
         <is>
-          <t>Nút In trên trang xem trước</t>
+          <t>In một phiếu</t>
         </is>
       </c>
       <c r="E95" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F95" s="15" t="inlineStr">
         <is>
-          <t>Đang ở trang xem trước bản in.</t>
+          <t>Phiếu đã điền đủ nguyên nhân và hành động.</t>
         </is>
       </c>
       <c r="G95" s="15" t="inlineStr">
         <is>
-          <t>1. Quan sát vị trí nút In
-2. Bấm nút In</t>
+          <t>1. Bấm In ở dòng phiếu
+2. Xem trang xem trước</t>
         </is>
       </c>
       <c r="H95" s="15" t="inlineStr">
@@ -6044,8 +6043,11 @@
       </c>
       <c r="I95" s="15" t="inlineStr">
         <is>
-          <t>- Nút In nằm bên phải, thẳng mép phải tờ giấy
-- Mở hộp thoại in của trình duyệt, bản xem không có nút In và không có khung viền</t>
+          <t>- Mở cửa sổ “Xem trước phiếu xử lý yêu cầu” ngay trên màn hình, không mở tab mới
+- Đầu bản in có tiêu đề công ty (logo, địa chỉ, điện thoại)
+- Bảng chi tiết có đủ 9 cột, trong đó có Nguyên nhân và Hành động
+- Có số phiếu xử lý, số phiếu yêu cầu, người yêu cầu, ngày nhận yêu cầu
+- Không còn chỗ nào bỏ trống dạng ký hiệu chờ điền</t>
         </is>
       </c>
       <c r="J95" s="15" t="inlineStr"/>
@@ -6069,30 +6071,77 @@
       <c r="P95" s="16" t="inlineStr"/>
       <c r="Q95" s="16" t="inlineStr"/>
     </row>
-    <row r="96" ht="26" customHeight="1">
-      <c r="A96" s="13" t="n"/>
-      <c r="B96" s="13" t="n"/>
-      <c r="C96" s="14" t="inlineStr">
-        <is>
-          <t>VIII. RÀNG BUỘC NHẬP LIỆU</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="n"/>
-      <c r="E96" s="4" t="n"/>
-      <c r="F96" s="4" t="n"/>
-      <c r="G96" s="4" t="n"/>
-      <c r="H96" s="4" t="n"/>
-      <c r="I96" s="4" t="n"/>
-      <c r="J96" s="4" t="n"/>
-      <c r="K96" s="4" t="n"/>
-      <c r="L96" s="4" t="n"/>
-      <c r="M96" s="4" t="n"/>
-      <c r="N96" s="4" t="n"/>
-      <c r="O96" s="4" t="n"/>
-      <c r="P96" s="4" t="n"/>
-      <c r="Q96" s="5" t="n"/>
-    </row>
-    <row r="97" ht="34" customHeight="1">
+    <row r="96" ht="69" customHeight="1">
+      <c r="A96" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>XUẤT EXCEL / IN</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>TC_07.004</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
+        <is>
+          <t>In danh sách theo bộ lọc</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F96" s="15" t="inlineStr">
+        <is>
+          <t>Đang lọc trạng thái “Đã tư vấn điện thoại”.</t>
+        </is>
+      </c>
+      <c r="G96" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm In danh sách
+2. Xem trang xem trước</t>
+        </is>
+      </c>
+      <c r="H96" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I96" s="15" t="inlineStr">
+        <is>
+          <t>- Mở cửa sổ “Xem trước danh sách phiếu xử lý yêu cầu”
+- Bảng chứa đúng các phiếu đang lọc, đủ 10 cột (có Người xử lý và Ngày xử lý)
+- Có 2 dòng “Thời gian” và “Phòng xử lý yêu cầu”; không lọc thì ghi “Tất cả”</t>
+        </is>
+      </c>
+      <c r="J96" s="15" t="inlineStr"/>
+      <c r="K96" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L96" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M96" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N96" s="15" t="inlineStr"/>
+      <c r="O96" s="16" t="inlineStr"/>
+      <c r="P96" s="16" t="inlineStr"/>
+      <c r="Q96" s="16" t="inlineStr"/>
+    </row>
+    <row r="97" ht="42" customHeight="1">
       <c r="A97" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -6100,32 +6149,33 @@
       </c>
       <c r="B97" s="15" t="inlineStr">
         <is>
-          <t>RÀNG BUỘC NHẬP LIỆU</t>
+          <t>XUẤT EXCEL / IN</t>
         </is>
       </c>
       <c r="C97" s="16" t="inlineStr">
         <is>
-          <t>TC_08.001</t>
+          <t>TC_07.005</t>
         </is>
       </c>
       <c r="D97" s="15" t="inlineStr">
         <is>
-          <t>Gửi đi khi thiếu Nguyên nhân và Hành động</t>
+          <t>Nút In trên trang xem trước</t>
         </is>
       </c>
       <c r="E97" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F97" s="15" t="inlineStr">
         <is>
-          <t>Phiếu có 1 thiết bị, chưa chọn gì.</t>
+          <t>Đang ở trang xem trước bản in.</t>
         </is>
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu và gửi, xác nhận</t>
+          <t>1. Quan sát vị trí nút In
+2. Bấm nút In</t>
         </is>
       </c>
       <c r="H97" s="15" t="inlineStr">
@@ -6135,8 +6185,8 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>- Không gửi được
-- Báo lỗi đỏ ngay dưới ô Nguyên nhân và ô Hành động của đúng dòng</t>
+          <t>- Nút In nằm ở góc trái trên cửa sổ xem trước
+- Mở hộp thoại in của trình duyệt, bản xem không có nút In và không có khung viền</t>
         </is>
       </c>
       <c r="J97" s="15" t="inlineStr"/>
@@ -6160,7 +6210,7 @@
       <c r="P97" s="16" t="inlineStr"/>
       <c r="Q97" s="16" t="inlineStr"/>
     </row>
-    <row r="98" ht="34" customHeight="1">
+    <row r="98" ht="75" customHeight="1">
       <c r="A98" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -6168,17 +6218,17 @@
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>RÀNG BUỘC NHẬP LIỆU</t>
+          <t>XUẤT EXCEL / IN</t>
         </is>
       </c>
       <c r="C98" s="16" t="inlineStr">
         <is>
-          <t>TC_08.002</t>
+          <t>TC_07.006</t>
         </is>
       </c>
       <c r="D98" s="15" t="inlineStr">
         <is>
-          <t>Tư vấn điện thoại thiếu nội dung xử lý</t>
+          <t>In danh sách khi chưa lọc gì — vượt trần in</t>
         </is>
       </c>
       <c r="E98" s="16" t="inlineStr">
@@ -6188,12 +6238,13 @@
       </c>
       <c r="F98" s="15" t="inlineStr">
         <is>
-          <t>Đã chọn nguyên nhân và hành động “Tư vấn điện thoại”, để trống nội dung xử lý.</t>
+          <t>Không áp bộ lọc nào, tổng hơn 5.000 phiếu.</t>
         </is>
       </c>
       <c r="G98" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu và gửi, xác nhận</t>
+          <t>1. Bấm In danh sách
+2. Đọc nội dung cửa sổ xem trước</t>
         </is>
       </c>
       <c r="H98" s="15" t="inlineStr">
@@ -6203,7 +6254,9 @@
       </c>
       <c r="I98" s="15" t="inlineStr">
         <is>
-          <t>- Chặn, báo lỗi đỏ dưới ô nội dung xử lý của đúng dòng</t>
+          <t>- ⚠️ KHÔNG dựng bản in; cửa sổ chỉ hiện lời nhắc nền vàng: danh sách vượt mức in tối đa 2.000 dòng, đề nghị thu hẹp bộ lọc hoặc dùng Xuất Excel
+- Lời nhắc ghi rõ số dòng thực tế
+- Trình duyệt không treo, không mở hộp thoại in</t>
         </is>
       </c>
       <c r="J98" s="15" t="inlineStr"/>
@@ -6227,7 +6280,7 @@
       <c r="P98" s="16" t="inlineStr"/>
       <c r="Q98" s="16" t="inlineStr"/>
     </row>
-    <row r="99" ht="34" customHeight="1">
+    <row r="99" ht="51" customHeight="1">
       <c r="A99" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -6235,33 +6288,33 @@
       </c>
       <c r="B99" s="15" t="inlineStr">
         <is>
-          <t>RÀNG BUỘC NHẬP LIỆU</t>
+          <t>XUẤT EXCEL / IN</t>
         </is>
       </c>
       <c r="C99" s="16" t="inlineStr">
         <is>
-          <t>TC_08.003</t>
+          <t>TC_07.007</t>
         </is>
       </c>
       <c r="D99" s="15" t="inlineStr">
         <is>
-          <t>Chọn trùng nguyên nhân cho cùng một thiết bị</t>
+          <t>Dòng tiến độ khi xuất Excel danh sách lớn</t>
         </is>
       </c>
       <c r="E99" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F99" s="15" t="inlineStr">
         <is>
-          <t>Phiếu có 2 dòng cùng hàng hóa, cùng serial.</t>
+          <t>Bộ lọc ra hơn 4.000 phiếu.</t>
         </is>
       </c>
       <c r="G99" s="15" t="inlineStr">
         <is>
-          <t>1. Chọn cho 2 dòng ít nhất một nguyên nhân giống nhau
-2. Bấm Lưu và gửi, xác nhận</t>
+          <t>1. Bấm Xuất Excel rồi Xuất file
+2. Quan sát dòng chữ cạnh nút trong lúc chờ</t>
         </is>
       </c>
       <c r="H99" s="15" t="inlineStr">
@@ -6271,7 +6324,9 @@
       </c>
       <c r="I99" s="15" t="inlineStr">
         <is>
-          <t>- Chặn, báo “Bị trùng nguyên nhân của cùng thiết bị” ở CẢ HAI dòng</t>
+          <t>- Hiện dòng “Đã tải …/… dòng”, sau đó “Đang dựng file …/… dòng”
+- Nút Xuất Excel khoá trong lúc chạy, xong thì mở lại
+- Tệp đủ số dòng, không thiếu trang</t>
         </is>
       </c>
       <c r="J99" s="15" t="inlineStr"/>
@@ -6295,7 +6350,7 @@
       <c r="P99" s="16" t="inlineStr"/>
       <c r="Q99" s="16" t="inlineStr"/>
     </row>
-    <row r="100" ht="34" customHeight="1">
+    <row r="100" ht="90" customHeight="1">
       <c r="A100" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -6303,33 +6358,33 @@
       </c>
       <c r="B100" s="15" t="inlineStr">
         <is>
-          <t>RÀNG BUỘC NHẬP LIỆU</t>
+          <t>XUẤT EXCEL / IN</t>
         </is>
       </c>
       <c r="C100" s="16" t="inlineStr">
         <is>
-          <t>TC_08.004</t>
+          <t>TC_07.008</t>
         </is>
       </c>
       <c r="D100" s="15" t="inlineStr">
         <is>
-          <t>Thiết bị tự gõ chưa chọn hàng hóa tương đương</t>
+          <t>Danh sách trường xuất file</t>
         </is>
       </c>
       <c r="E100" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F100" s="15" t="inlineStr">
         <is>
-          <t>Phiếu có dòng thiết bị người dùng tự gõ, chưa gắn hàng hóa.</t>
+          <t>Cửa sổ chọn trường xuất đang mở.</t>
         </is>
       </c>
       <c r="G100" s="15" t="inlineStr">
         <is>
-          <t>1. Chọn nguyên nhân + hành động cho dòng đó
-2. Bấm Lưu và gửi, xác nhận</t>
+          <t>1. Bấm Chọn tất cả
+2. Đếm số trường</t>
         </is>
       </c>
       <c r="H100" s="15" t="inlineStr">
@@ -6339,7 +6394,8 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>- Chặn, báo “Phải chọn hàng hóa tương đương” tại đúng dòng</t>
+          <t>- Có 14 trường: Số phiếu xử lý, Số phiếu yêu cầu, Khách hàng, Tên thiết bị liên quan, Người yêu cầu, Ngày nhận yêu cầu, Người xử lý, Ngày xử lý, Trạng thái, Địa chỉ sửa chữa, Ghi chú, Ngày tạo, Người cập nhật, Ngày cập nhật
+- Bỏ chọn hết thì nút Xuất file không dùng được</t>
         </is>
       </c>
       <c r="J100" s="15" t="inlineStr"/>
@@ -6363,72 +6419,28 @@
       <c r="P100" s="16" t="inlineStr"/>
       <c r="Q100" s="16" t="inlineStr"/>
     </row>
-    <row r="101" ht="34" customHeight="1">
-      <c r="A101" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B101" s="15" t="inlineStr">
-        <is>
-          <t>RÀNG BUỘC NHẬP LIỆU</t>
-        </is>
-      </c>
-      <c r="C101" s="16" t="inlineStr">
-        <is>
-          <t>TC_08.005</t>
-        </is>
-      </c>
-      <c r="D101" s="15" t="inlineStr">
-        <is>
-          <t>Gửi đi khi không có thiết bị nào</t>
-        </is>
-      </c>
-      <c r="E101" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F101" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu đã xóa hết dòng thiết bị.</t>
-        </is>
-      </c>
-      <c r="G101" s="15" t="inlineStr">
-        <is>
-          <t>1. Bấm Lưu và gửi, xác nhận</t>
-        </is>
-      </c>
-      <c r="H101" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I101" s="15" t="inlineStr">
-        <is>
-          <t>- Chặn, báo yêu cầu phải có ít nhất 1 thiết bị</t>
-        </is>
-      </c>
-      <c r="J101" s="15" t="inlineStr"/>
-      <c r="K101" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L101" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M101" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N101" s="15" t="inlineStr"/>
-      <c r="O101" s="16" t="inlineStr"/>
-      <c r="P101" s="16" t="inlineStr"/>
-      <c r="Q101" s="16" t="inlineStr"/>
+    <row r="101" ht="26" customHeight="1">
+      <c r="A101" s="13" t="n"/>
+      <c r="B101" s="13" t="n"/>
+      <c r="C101" s="14" t="inlineStr">
+        <is>
+          <t>VIII. RÀNG BUỘC NHẬP LIỆU</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="n"/>
+      <c r="E101" s="4" t="n"/>
+      <c r="F101" s="4" t="n"/>
+      <c r="G101" s="4" t="n"/>
+      <c r="H101" s="4" t="n"/>
+      <c r="I101" s="4" t="n"/>
+      <c r="J101" s="4" t="n"/>
+      <c r="K101" s="4" t="n"/>
+      <c r="L101" s="4" t="n"/>
+      <c r="M101" s="4" t="n"/>
+      <c r="N101" s="4" t="n"/>
+      <c r="O101" s="4" t="n"/>
+      <c r="P101" s="4" t="n"/>
+      <c r="Q101" s="5" t="n"/>
     </row>
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="15" t="inlineStr">
@@ -6443,27 +6455,27 @@
       </c>
       <c r="C102" s="16" t="inlineStr">
         <is>
-          <t>TC_08.006</t>
+          <t>TC_08.001</t>
         </is>
       </c>
       <c r="D102" s="15" t="inlineStr">
         <is>
-          <t>Lưu nháp không đòi nguyên nhân</t>
+          <t>Gửi đi khi thiếu Nguyên nhân và Hành động</t>
         </is>
       </c>
       <c r="E102" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F102" s="15" t="inlineStr">
         <is>
-          <t>Màn lập phiếu, chưa chọn gì.</t>
+          <t>Phiếu có 1 thiết bị, chưa chọn gì.</t>
         </is>
       </c>
       <c r="G102" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm Lưu nháp</t>
+          <t>1. Bấm Lưu và gửi, xác nhận</t>
         </is>
       </c>
       <c r="H102" s="15" t="inlineStr">
@@ -6473,8 +6485,8 @@
       </c>
       <c r="I102" s="15" t="inlineStr">
         <is>
-          <t>- Lưu thành công
-- ⚠️ Ràng buộc nguyên nhân/hành động chỉ áp dụng khi gửi đi</t>
+          <t>- Không gửi được
+- Báo lỗi đỏ ngay dưới ô Nguyên nhân và ô Hành động của đúng dòng</t>
         </is>
       </c>
       <c r="J102" s="15" t="inlineStr"/>
@@ -6511,38 +6523,37 @@
       </c>
       <c r="C103" s="16" t="inlineStr">
         <is>
-          <t>TC_08.007</t>
+          <t>TC_08.002</t>
         </is>
       </c>
       <c r="D103" s="15" t="inlineStr">
         <is>
-          <t>Ô chỉ đọc không gõ được</t>
+          <t>Tư vấn điện thoại thiếu nội dung xử lý</t>
         </is>
       </c>
       <c r="E103" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F103" s="15" t="inlineStr">
         <is>
-          <t>Màn lập phiếu.</t>
+          <t>Đã chọn nguyên nhân và hành động “Tư vấn điện thoại”, để trống nội dung xử lý.</t>
         </is>
       </c>
       <c r="G103" s="15" t="inlineStr">
         <is>
-          <t>1. Bấm vào các ô của khối Thông tin yêu cầu, thử gõ</t>
+          <t>1. Bấm Lưu và gửi, xác nhận</t>
         </is>
       </c>
       <c r="H103" s="15" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I103" s="15" t="inlineStr">
         <is>
-          <t>- Không gõ được vào bất kỳ ô nào trong khối này
-- Ô có nền xám phân biệt với ô nhập được</t>
+          <t>- Chặn, báo lỗi đỏ dưới ô nội dung xử lý của đúng dòng</t>
         </is>
       </c>
       <c r="J103" s="15" t="inlineStr"/>
@@ -6566,28 +6577,73 @@
       <c r="P103" s="16" t="inlineStr"/>
       <c r="Q103" s="16" t="inlineStr"/>
     </row>
-    <row r="104" ht="26" customHeight="1">
-      <c r="A104" s="13" t="n"/>
-      <c r="B104" s="13" t="n"/>
-      <c r="C104" s="14" t="inlineStr">
-        <is>
-          <t>IX. CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="n"/>
-      <c r="E104" s="4" t="n"/>
-      <c r="F104" s="4" t="n"/>
-      <c r="G104" s="4" t="n"/>
-      <c r="H104" s="4" t="n"/>
-      <c r="I104" s="4" t="n"/>
-      <c r="J104" s="4" t="n"/>
-      <c r="K104" s="4" t="n"/>
-      <c r="L104" s="4" t="n"/>
-      <c r="M104" s="4" t="n"/>
-      <c r="N104" s="4" t="n"/>
-      <c r="O104" s="4" t="n"/>
-      <c r="P104" s="4" t="n"/>
-      <c r="Q104" s="5" t="n"/>
+    <row r="104" ht="34" customHeight="1">
+      <c r="A104" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>RÀNG BUỘC NHẬP LIỆU</t>
+        </is>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>TC_08.003</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>Chọn trùng nguyên nhân cho cùng một thiết bị</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F104" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu có 2 dòng cùng hàng hóa, cùng serial.</t>
+        </is>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>1. Chọn cho 2 dòng ít nhất một nguyên nhân giống nhau
+2. Bấm Lưu và gửi, xác nhận</t>
+        </is>
+      </c>
+      <c r="H104" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>- Chặn, báo “Bị trùng nguyên nhân của cùng thiết bị” ở CẢ HAI dòng</t>
+        </is>
+      </c>
+      <c r="J104" s="15" t="inlineStr"/>
+      <c r="K104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N104" s="15" t="inlineStr"/>
+      <c r="O104" s="16" t="inlineStr"/>
+      <c r="P104" s="16" t="inlineStr"/>
+      <c r="Q104" s="16" t="inlineStr"/>
     </row>
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="15" t="inlineStr">
@@ -6597,33 +6653,33 @@
       </c>
       <c r="B105" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU</t>
         </is>
       </c>
       <c r="C105" s="16" t="inlineStr">
         <is>
-          <t>TC_09.001</t>
+          <t>TC_08.004</t>
         </is>
       </c>
       <c r="D105" s="15" t="inlineStr">
         <is>
-          <t>Hai người cùng xử lý một phiếu</t>
+          <t>Thiết bị tự gõ chưa chọn hàng hóa tương đương</t>
         </is>
       </c>
       <c r="E105" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F105" s="15" t="inlineStr">
         <is>
-          <t>Phiếu “Chờ CCTT”, hai người E và F cùng có quyền và cùng mở phiếu.</t>
+          <t>Phiếu có dòng thiết bị người dùng tự gõ, chưa gắn hàng hóa.</t>
         </is>
       </c>
       <c r="G105" s="15" t="inlineStr">
         <is>
-          <t>1. E bấm Không duyệt kèm lý do
-2. F (chưa tải lại trang) cũng bấm Không duyệt</t>
+          <t>1. Chọn nguyên nhân + hành động cho dòng đó
+2. Bấm Lưu và gửi, xác nhận</t>
         </is>
       </c>
       <c r="H105" s="15" t="inlineStr">
@@ -6633,8 +6689,7 @@
       </c>
       <c r="I105" s="15" t="inlineStr">
         <is>
-          <t>- Thao tác của F bị chặn, báo phiếu không ở trạng thái Chờ CCTT
-- Không treo trang</t>
+          <t>- Chặn, báo “Phải chọn hàng hóa tương đương” tại đúng dòng</t>
         </is>
       </c>
       <c r="J105" s="15" t="inlineStr"/>
@@ -6666,33 +6721,32 @@
       </c>
       <c r="B106" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU</t>
         </is>
       </c>
       <c r="C106" s="16" t="inlineStr">
         <is>
-          <t>TC_09.002</t>
+          <t>TC_08.005</t>
         </is>
       </c>
       <c r="D106" s="15" t="inlineStr">
         <is>
-          <t>Xóa phiếu vừa bị người khác xóa</t>
+          <t>Gửi đi khi không có thiết bị nào</t>
         </is>
       </c>
       <c r="E106" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F106" s="15" t="inlineStr">
         <is>
-          <t>Hai cửa sổ cùng mở danh sách, cùng thấy phiếu nháp X.</t>
+          <t>Phiếu đã xóa hết dòng thiết bị.</t>
         </is>
       </c>
       <c r="G106" s="15" t="inlineStr">
         <is>
-          <t>1. Cửa sổ 1 xóa phiếu X
-2. Cửa sổ 2 (chưa tải lại) cũng bấm Xóa phiếu X</t>
+          <t>1. Bấm Lưu và gửi, xác nhận</t>
         </is>
       </c>
       <c r="H106" s="15" t="inlineStr">
@@ -6702,7 +6756,7 @@
       </c>
       <c r="I106" s="15" t="inlineStr">
         <is>
-          <t>- Cửa sổ 2 báo dữ liệu đã thay đổi, không treo trang</t>
+          <t>- Chặn, báo yêu cầu phải có ít nhất 1 thiết bị</t>
         </is>
       </c>
       <c r="J106" s="15" t="inlineStr"/>
@@ -6734,43 +6788,43 @@
       </c>
       <c r="B107" s="15" t="inlineStr">
         <is>
-          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+          <t>RÀNG BUỘC NHẬP LIỆU</t>
         </is>
       </c>
       <c r="C107" s="16" t="inlineStr">
         <is>
-          <t>TC_09.003</t>
+          <t>TC_08.006</t>
         </is>
       </c>
       <c r="D107" s="15" t="inlineStr">
         <is>
-          <t>Dữ liệu lập bên ERP hiện ngay bên đây</t>
+          <t>Lưu nháp không đòi nguyên nhân</t>
         </is>
       </c>
       <c r="E107" s="16" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F107" s="15" t="inlineStr">
         <is>
-          <t>Có tài khoản dùng được cả 2 cổng.</t>
+          <t>Màn lập phiếu, chưa chọn gì.</t>
         </is>
       </c>
       <c r="G107" s="15" t="inlineStr">
         <is>
-          <t>1. Lập 1 phiếu xử lý bên phần mềm ERP
-2. Sang màn hình này, tìm theo số phiếu vừa lập</t>
+          <t>1. Bấm Lưu nháp</t>
         </is>
       </c>
       <c r="H107" s="15" t="inlineStr">
         <is>
-          <t>Số phiếu vừa lập bên ERP</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I107" s="15" t="inlineStr">
         <is>
-          <t>- Tìm thấy đúng phiếu, mở ra thấy đủ nguyên nhân và hành động đã chọn bên ERP</t>
+          <t>- Lưu thành công
+- ⚠️ Ràng buộc nguyên nhân/hành động chỉ áp dụng khi gửi đi</t>
         </is>
       </c>
       <c r="J107" s="15" t="inlineStr"/>
@@ -6794,149 +6848,143 @@
       <c r="P107" s="16" t="inlineStr"/>
       <c r="Q107" s="16" t="inlineStr"/>
     </row>
-    <row r="108" ht="26" customHeight="1">
-      <c r="A108" s="13" t="n"/>
-      <c r="B108" s="13" t="n"/>
-      <c r="C108" s="14" t="inlineStr">
-        <is>
-          <t>X. LỊCH SỬ THAY ĐỔI</t>
-        </is>
-      </c>
-      <c r="D108" s="4" t="n"/>
-      <c r="E108" s="4" t="n"/>
-      <c r="F108" s="4" t="n"/>
-      <c r="G108" s="4" t="n"/>
-      <c r="H108" s="4" t="n"/>
-      <c r="I108" s="4" t="n"/>
-      <c r="J108" s="4" t="n"/>
-      <c r="K108" s="4" t="n"/>
-      <c r="L108" s="4" t="n"/>
-      <c r="M108" s="4" t="n"/>
-      <c r="N108" s="4" t="n"/>
-      <c r="O108" s="4" t="n"/>
-      <c r="P108" s="4" t="n"/>
-      <c r="Q108" s="5" t="n"/>
-    </row>
-    <row r="109" ht="64" customHeight="1">
-      <c r="A109" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B109" s="15" t="inlineStr">
-        <is>
-          <t>LỊCH SỬ THAY ĐỔI</t>
-        </is>
-      </c>
-      <c r="C109" s="16" t="inlineStr">
-        <is>
-          <t>TC_10.001</t>
-        </is>
-      </c>
-      <c r="D109" s="15" t="inlineStr">
-        <is>
-          <t>Lịch sử ghi nhận đủ các thao tác</t>
-        </is>
-      </c>
-      <c r="E109" s="16" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="F109" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu vừa trải qua: lập mới → sửa và gửi đi → bị Không duyệt.</t>
-        </is>
-      </c>
-      <c r="G109" s="15" t="inlineStr">
-        <is>
-          <t>1. Mở menu hành động của phiếu, bấm Lịch sử
-2. Đọc các mốc từ trên xuống</t>
-        </is>
-      </c>
-      <c r="H109" s="15" t="inlineStr">
+    <row r="108" ht="34" customHeight="1">
+      <c r="A108" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>RÀNG BUỘC NHẬP LIỆU</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="inlineStr">
+        <is>
+          <t>TC_08.007</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>Ô chỉ đọc không gõ được</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>Màn lập phiếu.</t>
+        </is>
+      </c>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>1. Bấm vào các ô của khối Thông tin yêu cầu, thử gõ</t>
+        </is>
+      </c>
+      <c r="H108" s="15" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="I108" s="15" t="inlineStr">
+        <is>
+          <t>- Không gõ được vào bất kỳ ô nào trong khối này
+- Ô có nền xám phân biệt với ô nhập được</t>
+        </is>
+      </c>
+      <c r="J108" s="15" t="inlineStr"/>
+      <c r="K108" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L108" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M108" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N108" s="15" t="inlineStr"/>
+      <c r="O108" s="16" t="inlineStr"/>
+      <c r="P108" s="16" t="inlineStr"/>
+      <c r="Q108" s="16" t="inlineStr"/>
+    </row>
+    <row r="109" ht="26" customHeight="1">
+      <c r="A109" s="13" t="n"/>
+      <c r="B109" s="13" t="n"/>
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>IX. CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="n"/>
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="4" t="n"/>
+      <c r="H109" s="4" t="n"/>
+      <c r="I109" s="4" t="n"/>
+      <c r="J109" s="4" t="n"/>
+      <c r="K109" s="4" t="n"/>
+      <c r="L109" s="4" t="n"/>
+      <c r="M109" s="4" t="n"/>
+      <c r="N109" s="4" t="n"/>
+      <c r="O109" s="4" t="n"/>
+      <c r="P109" s="4" t="n"/>
+      <c r="Q109" s="5" t="n"/>
+    </row>
+    <row r="110" ht="34" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
+        </is>
+      </c>
+      <c r="C110" s="16" t="inlineStr">
+        <is>
+          <t>TC_09.001</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="inlineStr">
+        <is>
+          <t>Hai người cùng xử lý một phiếu</t>
+        </is>
+      </c>
+      <c r="E110" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F110" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu “Chờ CCTT”, hai người E và F cùng có quyền và cùng mở phiếu.</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="inlineStr">
+        <is>
+          <t>1. E bấm Không duyệt kèm lý do
+2. F (chưa tải lại trang) cũng bấm Không duyệt</t>
+        </is>
+      </c>
+      <c r="H110" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I109" s="15" t="inlineStr">
-        <is>
-          <t>- Danh sách sắp xếp MỚI → CŨ
-- Có đủ 3 mốc: Từ chối · Thay đổi thông tin · Tạo mới
-- Mỗi mốc hiện: thời gian, tên hành động, người thực hiện kèm phòng ban
-- Mốc Từ chối hiện ĐÚNG lý do đã nhập</t>
-        </is>
-      </c>
-      <c r="J109" s="15" t="inlineStr"/>
-      <c r="K109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M109" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N109" s="15" t="inlineStr"/>
-      <c r="O109" s="16" t="inlineStr"/>
-      <c r="P109" s="16" t="inlineStr"/>
-      <c r="Q109" s="16" t="inlineStr"/>
-    </row>
-    <row r="110" ht="69" customHeight="1">
-      <c r="A110" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B110" s="15" t="inlineStr">
-        <is>
-          <t>LỊCH SỬ THAY ĐỔI</t>
-        </is>
-      </c>
-      <c r="C110" s="16" t="inlineStr">
-        <is>
-          <t>TC_10.002</t>
-        </is>
-      </c>
-      <c r="D110" s="15" t="inlineStr">
-        <is>
-          <t>Bộ lọc trong Lịch sử</t>
-        </is>
-      </c>
-      <c r="E110" s="16" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F110" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu có nhiều mốc lịch sử.</t>
-        </is>
-      </c>
-      <c r="G110" s="15" t="inlineStr">
-        <is>
-          <t>1. Mở popup Lịch sử
-2. Mở ô Loại hành động
-3. Chọn “Thay đổi trạng thái”
-4. Bấm Tìm kiếm</t>
-        </is>
-      </c>
-      <c r="H110" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I110" s="15" t="inlineStr">
         <is>
-          <t>- Ô Loại hành động có đúng 3 lựa chọn: Tạo mới · Thay đổi thông tin · Thay đổi trạng thái
-- Ô Người thực hiện liệt kê đầy đủ nhân sự, không chỉ vài người có trong log
-- Lọc xong chỉ còn mốc thuộc nhóm đã chọn</t>
+          <t>- Thao tác của F bị chặn, báo phiếu không ở trạng thái Chờ CCTT
+- Không treo trang</t>
         </is>
       </c>
       <c r="J110" s="15" t="inlineStr"/>
@@ -6968,33 +7016,33 @@
       </c>
       <c r="B111" s="15" t="inlineStr">
         <is>
-          <t>LỊCH SỬ THAY ĐỔI</t>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
         </is>
       </c>
       <c r="C111" s="16" t="inlineStr">
         <is>
-          <t>TC_10.003</t>
+          <t>TC_09.002</t>
         </is>
       </c>
       <c r="D111" s="15" t="inlineStr">
         <is>
-          <t>Lịch sử ở màn chi tiết giống popup ngoài danh sách</t>
+          <t>Xóa phiếu vừa bị người khác xóa</t>
         </is>
       </c>
       <c r="E111" s="16" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="F111" s="15" t="inlineStr">
         <is>
-          <t>Cùng một phiếu.</t>
+          <t>Hai cửa sổ cùng mở danh sách, cùng thấy phiếu nháp X.</t>
         </is>
       </c>
       <c r="G111" s="15" t="inlineStr">
         <is>
-          <t>1. Mở popup Lịch sử từ danh sách, ghi lại nội dung
-2. Mở màn chi tiết, mở khối Lịch sử</t>
+          <t>1. Cửa sổ 1 xóa phiếu X
+2. Cửa sổ 2 (chưa tải lại) cũng bấm Xóa phiếu X</t>
         </is>
       </c>
       <c r="H111" s="15" t="inlineStr">
@@ -7004,7 +7052,7 @@
       </c>
       <c r="I111" s="15" t="inlineStr">
         <is>
-          <t>- Hai nơi hiện cùng số mốc, cùng nội dung, cùng thứ tự, cùng bộ lọc</t>
+          <t>- Cửa sổ 2 báo dữ liệu đã thay đổi, không treo trang</t>
         </is>
       </c>
       <c r="J111" s="15" t="inlineStr"/>
@@ -7028,7 +7076,7 @@
       <c r="P111" s="16" t="inlineStr"/>
       <c r="Q111" s="16" t="inlineStr"/>
     </row>
-    <row r="112" ht="55" customHeight="1">
+    <row r="112" ht="34" customHeight="1">
       <c r="A112" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -7036,43 +7084,43 @@
       </c>
       <c r="B112" s="15" t="inlineStr">
         <is>
-          <t>LỊCH SỬ THAY ĐỔI</t>
+          <t>CÔ LẬP DỮ LIỆU &amp; THAO TÁC ĐỒNG THỜI</t>
         </is>
       </c>
       <c r="C112" s="16" t="inlineStr">
         <is>
-          <t>TC_10.004</t>
+          <t>TC_09.003</t>
         </is>
       </c>
       <c r="D112" s="15" t="inlineStr">
         <is>
-          <t>Lịch sử không ghi nhiễu khi chỉ đổi dòng thiết bị</t>
+          <t>Dữ liệu lập bên ERP hiện ngay bên đây</t>
         </is>
       </c>
       <c r="E112" s="16" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F112" s="15" t="inlineStr">
         <is>
-          <t>Phiếu nháp có 2 dòng thiết bị.</t>
+          <t>Có tài khoản dùng được cả 2 cổng.</t>
         </is>
       </c>
       <c r="G112" s="15" t="inlineStr">
         <is>
-          <t>1. Sửa phiếu, chỉ đổi nguyên nhân của một dòng rồi Lưu nháp
-2. Mở Lịch sử</t>
+          <t>1. Lập 1 phiếu xử lý bên phần mềm ERP
+2. Sang màn hình này, tìm theo số phiếu vừa lập</t>
         </is>
       </c>
       <c r="H112" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Số phiếu vừa lập bên ERP</t>
         </is>
       </c>
       <c r="I112" s="15" t="inlineStr">
         <is>
-          <t>- ⚠️ Lịch sử KHÔNG ghi nhận thay đổi ở dòng thiết bị (hiện chỉ theo dõi thông tin chung của phiếu và trạng thái) — đây là giới hạn đã biết, không phải lỗi mất dữ liệu</t>
+          <t>- Tìm thấy đúng phiếu, mở ra thấy đủ nguyên nhân và hành động đã chọn bên ERP</t>
         </is>
       </c>
       <c r="J112" s="15" t="inlineStr"/>
@@ -7101,7 +7149,7 @@
       <c r="B113" s="13" t="n"/>
       <c r="C113" s="14" t="inlineStr">
         <is>
-          <t>XI. LUỒNG NGHIỆP VỤ ĐẦU – CUỐI</t>
+          <t>X. LỊCH SỬ THAY ĐỔI</t>
         </is>
       </c>
       <c r="D113" s="4" t="n"/>
@@ -7119,7 +7167,7 @@
       <c r="P113" s="4" t="n"/>
       <c r="Q113" s="5" t="n"/>
     </row>
-    <row r="114" ht="96" customHeight="1">
+    <row r="114" ht="64" customHeight="1">
       <c r="A114" s="15" t="inlineStr">
         <is>
           <t>Phiếu xử lý yêu cầu</t>
@@ -7127,30 +7175,332 @@
       </c>
       <c r="B114" s="15" t="inlineStr">
         <is>
+          <t>LỊCH SỬ THAY ĐỔI</t>
+        </is>
+      </c>
+      <c r="C114" s="16" t="inlineStr">
+        <is>
+          <t>TC_10.001</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Lịch sử ghi nhận đủ các thao tác</t>
+        </is>
+      </c>
+      <c r="E114" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F114" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu vừa trải qua: lập mới → sửa và gửi đi → bị Không duyệt.</t>
+        </is>
+      </c>
+      <c r="G114" s="15" t="inlineStr">
+        <is>
+          <t>1. Mở menu hành động của phiếu, bấm Lịch sử
+2. Đọc các mốc từ trên xuống</t>
+        </is>
+      </c>
+      <c r="H114" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I114" s="15" t="inlineStr">
+        <is>
+          <t>- Danh sách sắp xếp MỚI → CŨ
+- Có đủ 3 mốc: Từ chối · Thay đổi thông tin · Tạo mới
+- Mỗi mốc hiện: thời gian, tên hành động, người thực hiện kèm phòng ban
+- Mốc Từ chối hiện ĐÚNG lý do đã nhập</t>
+        </is>
+      </c>
+      <c r="J114" s="15" t="inlineStr"/>
+      <c r="K114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M114" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N114" s="15" t="inlineStr"/>
+      <c r="O114" s="16" t="inlineStr"/>
+      <c r="P114" s="16" t="inlineStr"/>
+      <c r="Q114" s="16" t="inlineStr"/>
+    </row>
+    <row r="115" ht="69" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="inlineStr">
+        <is>
+          <t>LỊCH SỬ THAY ĐỔI</t>
+        </is>
+      </c>
+      <c r="C115" s="16" t="inlineStr">
+        <is>
+          <t>TC_10.002</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>Bộ lọc trong Lịch sử</t>
+        </is>
+      </c>
+      <c r="E115" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F115" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu có nhiều mốc lịch sử.</t>
+        </is>
+      </c>
+      <c r="G115" s="15" t="inlineStr">
+        <is>
+          <t>1. Mở popup Lịch sử
+2. Mở ô Loại hành động
+3. Chọn “Thay đổi trạng thái”
+4. Bấm Tìm kiếm</t>
+        </is>
+      </c>
+      <c r="H115" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I115" s="15" t="inlineStr">
+        <is>
+          <t>- Ô Loại hành động có đúng 3 lựa chọn: Tạo mới · Thay đổi thông tin · Thay đổi trạng thái
+- Ô Người thực hiện liệt kê đầy đủ nhân sự, không chỉ vài người có trong log
+- Lọc xong chỉ còn mốc thuộc nhóm đã chọn</t>
+        </is>
+      </c>
+      <c r="J115" s="15" t="inlineStr"/>
+      <c r="K115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N115" s="15" t="inlineStr"/>
+      <c r="O115" s="16" t="inlineStr"/>
+      <c r="P115" s="16" t="inlineStr"/>
+      <c r="Q115" s="16" t="inlineStr"/>
+    </row>
+    <row r="116" ht="34" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>LỊCH SỬ THAY ĐỔI</t>
+        </is>
+      </c>
+      <c r="C116" s="16" t="inlineStr">
+        <is>
+          <t>TC_10.003</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>Lịch sử ở màn chi tiết giống popup ngoài danh sách</t>
+        </is>
+      </c>
+      <c r="E116" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F116" s="15" t="inlineStr">
+        <is>
+          <t>Cùng một phiếu.</t>
+        </is>
+      </c>
+      <c r="G116" s="15" t="inlineStr">
+        <is>
+          <t>1. Mở popup Lịch sử từ danh sách, ghi lại nội dung
+2. Mở màn chi tiết, mở khối Lịch sử</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I116" s="15" t="inlineStr">
+        <is>
+          <t>- Hai nơi hiện cùng số mốc, cùng nội dung, cùng thứ tự, cùng bộ lọc</t>
+        </is>
+      </c>
+      <c r="J116" s="15" t="inlineStr"/>
+      <c r="K116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M116" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N116" s="15" t="inlineStr"/>
+      <c r="O116" s="16" t="inlineStr"/>
+      <c r="P116" s="16" t="inlineStr"/>
+      <c r="Q116" s="16" t="inlineStr"/>
+    </row>
+    <row r="117" ht="55" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>LỊCH SỬ THAY ĐỔI</t>
+        </is>
+      </c>
+      <c r="C117" s="16" t="inlineStr">
+        <is>
+          <t>TC_10.004</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr">
+        <is>
+          <t>Lịch sử không ghi nhiễu khi chỉ đổi dòng thiết bị</t>
+        </is>
+      </c>
+      <c r="E117" s="16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F117" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu nháp có 2 dòng thiết bị.</t>
+        </is>
+      </c>
+      <c r="G117" s="15" t="inlineStr">
+        <is>
+          <t>1. Sửa phiếu, chỉ đổi nguyên nhân của một dòng rồi Lưu nháp
+2. Mở Lịch sử</t>
+        </is>
+      </c>
+      <c r="H117" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I117" s="15" t="inlineStr">
+        <is>
+          <t>- ⚠️ Lịch sử KHÔNG ghi nhận thay đổi ở dòng thiết bị (hiện chỉ theo dõi thông tin chung của phiếu và trạng thái) — đây là giới hạn đã biết, không phải lỗi mất dữ liệu</t>
+        </is>
+      </c>
+      <c r="J117" s="15" t="inlineStr"/>
+      <c r="K117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M117" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N117" s="15" t="inlineStr"/>
+      <c r="O117" s="16" t="inlineStr"/>
+      <c r="P117" s="16" t="inlineStr"/>
+      <c r="Q117" s="16" t="inlineStr"/>
+    </row>
+    <row r="118" ht="26" customHeight="1">
+      <c r="A118" s="13" t="n"/>
+      <c r="B118" s="13" t="n"/>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>XI. LUỒNG NGHIỆP VỤ ĐẦU – CUỐI</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="n"/>
+      <c r="E118" s="4" t="n"/>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n"/>
+      <c r="I118" s="4" t="n"/>
+      <c r="J118" s="4" t="n"/>
+      <c r="K118" s="4" t="n"/>
+      <c r="L118" s="4" t="n"/>
+      <c r="M118" s="4" t="n"/>
+      <c r="N118" s="4" t="n"/>
+      <c r="O118" s="4" t="n"/>
+      <c r="P118" s="4" t="n"/>
+      <c r="Q118" s="5" t="n"/>
+    </row>
+    <row r="119" ht="96" customHeight="1">
+      <c r="A119" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
           <t>LUỒNG NGHIỆP VỤ ĐẦU – CUỐI</t>
         </is>
       </c>
-      <c r="C114" s="16" t="inlineStr">
+      <c r="C119" s="16" t="inlineStr">
         <is>
           <t>TC_11.001</t>
         </is>
       </c>
-      <c r="D114" s="15" t="inlineStr">
+      <c r="D119" s="15" t="inlineStr">
         <is>
           <t>Luồng đầy đủ: lập → gửi → không duyệt → gửi lại → xóa</t>
         </is>
       </c>
-      <c r="E114" s="16" t="inlineStr">
+      <c r="E119" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F114" s="15" t="inlineStr">
+      <c r="F119" s="15" t="inlineStr">
         <is>
           <t>Phiếu yêu cầu Y đang “Chờ xử lý”. Nhân viên G thuộc phòng tiếp nhận, E có quyền tạo phiếu cung cấp thông tin.</t>
         </is>
       </c>
-      <c r="G114" s="15" t="inlineStr">
+      <c r="G119" s="15" t="inlineStr">
         <is>
           <t>1. G lập phiếu xử lý từ Y, chọn nguyên nhân + hành động Cung cấp thông tin, Lưu và gửi
 2. E nhận thông báo, mở phiếu, bấm Không duyệt kèm lý do
@@ -7159,12 +7509,12 @@
 5. Mở màn Yêu cầu kiểm tra sửa chữa – bảo hành, tìm phiếu Y</t>
         </is>
       </c>
-      <c r="H114" s="15" t="inlineStr">
+      <c r="H119" s="15" t="inlineStr">
         <is>
           <t>Lý do: “Thiếu thông tin báo giá”</t>
         </is>
       </c>
-      <c r="I114" s="15" t="inlineStr">
+      <c r="I119" s="15" t="inlineStr">
         <is>
           <t>- Bước 1: phiếu “Chờ CCTT”, phiếu Y thành “Đã xử lý”
 - Bước 2: phiếu về “Đang tạo”, phiếu Y VẪN “Đã xử lý”
@@ -7172,59 +7522,59 @@
 - Bước 4-5: xóa xong phiếu Y TRỞ LẠI “Chờ xử lý” và lại lập được phiếu xử lý mới</t>
         </is>
       </c>
-      <c r="J114" s="15" t="inlineStr"/>
-      <c r="K114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M114" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N114" s="15" t="inlineStr"/>
-      <c r="O114" s="16" t="inlineStr"/>
-      <c r="P114" s="16" t="inlineStr"/>
-      <c r="Q114" s="16" t="inlineStr"/>
-    </row>
-    <row r="115" ht="53" customHeight="1">
-      <c r="A115" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B115" s="15" t="inlineStr">
+      <c r="J119" s="15" t="inlineStr"/>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N119" s="15" t="inlineStr"/>
+      <c r="O119" s="16" t="inlineStr"/>
+      <c r="P119" s="16" t="inlineStr"/>
+      <c r="Q119" s="16" t="inlineStr"/>
+    </row>
+    <row r="120" ht="53" customHeight="1">
+      <c r="A120" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
         <is>
           <t>LUỒNG NGHIỆP VỤ ĐẦU – CUỐI</t>
         </is>
       </c>
-      <c r="C115" s="16" t="inlineStr">
+      <c r="C120" s="16" t="inlineStr">
         <is>
           <t>TC_11.002</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
+      <c r="D120" s="15" t="inlineStr">
         <is>
           <t>Luồng kết thúc bằng tư vấn điện thoại</t>
         </is>
       </c>
-      <c r="E115" s="16" t="inlineStr">
+      <c r="E120" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F115" s="15" t="inlineStr">
+      <c r="F120" s="15" t="inlineStr">
         <is>
           <t>Phiếu yêu cầu Z đang “Chờ xử lý”, có 1 thiết bị.</t>
         </is>
       </c>
-      <c r="G115" s="15" t="inlineStr">
+      <c r="G120" s="15" t="inlineStr">
         <is>
           <t>1. Lập phiếu xử lý từ Z
 2. Chọn nguyên nhân, hành động “Tư vấn điện thoại”, nhập nội dung xử lý
@@ -7232,12 +7582,12 @@
 4. Kiểm tra phiếu xử lý và phiếu Z</t>
         </is>
       </c>
-      <c r="H115" s="15" t="inlineStr">
+      <c r="H120" s="15" t="inlineStr">
         <is>
           <t>Nội dung xử lý: “Hướng dẫn khách tự khắc phục”</t>
         </is>
       </c>
-      <c r="I115" s="15" t="inlineStr">
+      <c r="I120" s="15" t="inlineStr">
         <is>
           <t>- Phiếu xử lý: “Đã tư vấn điện thoại”
 - Phiếu Z: “Đã tư vấn điện thoại”
@@ -7245,113 +7595,114 @@
 - Luồng dịch vụ kết thúc, không đi tiếp</t>
         </is>
       </c>
-      <c r="J115" s="15" t="inlineStr"/>
-      <c r="K115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M115" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N115" s="15" t="inlineStr"/>
-      <c r="O115" s="16" t="inlineStr"/>
-      <c r="P115" s="16" t="inlineStr"/>
-      <c r="Q115" s="16" t="inlineStr"/>
-    </row>
-    <row r="116" ht="34" customHeight="1">
-      <c r="A116" s="15" t="inlineStr">
-        <is>
-          <t>Phiếu xử lý yêu cầu</t>
-        </is>
-      </c>
-      <c r="B116" s="15" t="inlineStr">
+      <c r="J120" s="15" t="inlineStr"/>
+      <c r="K120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M120" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N120" s="15" t="inlineStr"/>
+      <c r="O120" s="16" t="inlineStr"/>
+      <c r="P120" s="16" t="inlineStr"/>
+      <c r="Q120" s="16" t="inlineStr"/>
+    </row>
+    <row r="121" ht="34" customHeight="1">
+      <c r="A121" s="15" t="inlineStr">
+        <is>
+          <t>Phiếu xử lý yêu cầu</t>
+        </is>
+      </c>
+      <c r="B121" s="15" t="inlineStr">
         <is>
           <t>LUỒNG NGHIỆP VỤ ĐẦU – CUỐI</t>
         </is>
       </c>
-      <c r="C116" s="16" t="inlineStr">
+      <c r="C121" s="16" t="inlineStr">
         <is>
           <t>TC_11.003</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
+      <c r="D121" s="15" t="inlineStr">
         <is>
           <t>Đối chiếu số liệu 2 cổng</t>
         </is>
       </c>
-      <c r="E116" s="16" t="inlineStr">
+      <c r="E121" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F116" s="15" t="inlineStr">
+      <c r="F121" s="15" t="inlineStr">
         <is>
           <t>Cùng bộ lọc trạng thái “Chờ CCTT” trên cả 2 cổng, cùng tài khoản.</t>
         </is>
       </c>
-      <c r="G116" s="15" t="inlineStr">
+      <c r="G121" s="15" t="inlineStr">
         <is>
           <t>1. Đếm số phiếu bên phần mềm ERP
 2. Đếm số phiếu trên màn hình này</t>
         </is>
       </c>
-      <c r="H116" s="15" t="inlineStr">
+      <c r="H121" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I116" s="15" t="inlineStr">
+      <c r="I121" s="15" t="inlineStr">
         <is>
           <t>- Hai con số bằng nhau (cùng đọc một nguồn dữ liệu)</t>
         </is>
       </c>
-      <c r="J116" s="15" t="inlineStr"/>
-      <c r="K116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="L116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M116" s="16" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N116" s="15" t="inlineStr"/>
-      <c r="O116" s="16" t="inlineStr"/>
-      <c r="P116" s="16" t="inlineStr"/>
-      <c r="Q116" s="16" t="inlineStr"/>
+      <c r="J121" s="15" t="inlineStr"/>
+      <c r="K121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="L121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N121" s="15" t="inlineStr"/>
+      <c r="O121" s="16" t="inlineStr"/>
+      <c r="P121" s="16" t="inlineStr"/>
+      <c r="Q121" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="44">
     <mergeCell ref="C113:Q113"/>
+    <mergeCell ref="C109:Q109"/>
     <mergeCell ref="B9:N9"/>
     <mergeCell ref="I15:J15"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="A11:E11"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="C31:Q31"/>
+    <mergeCell ref="C118:Q118"/>
     <mergeCell ref="B6:N6"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="C90:Q90"/>
     <mergeCell ref="B5:N5"/>
     <mergeCell ref="K11:L11"/>
     <mergeCell ref="M11:N11"/>
+    <mergeCell ref="C60:Q60"/>
     <mergeCell ref="B4:N4"/>
     <mergeCell ref="O12:Q12"/>
-    <mergeCell ref="C76:Q76"/>
     <mergeCell ref="B7:N7"/>
     <mergeCell ref="C39:Q39"/>
     <mergeCell ref="B3:N3"/>
@@ -7368,24 +7719,23 @@
     <mergeCell ref="C18:Q18"/>
     <mergeCell ref="K14:L14"/>
     <mergeCell ref="B2:N2"/>
-    <mergeCell ref="C96:Q96"/>
-    <mergeCell ref="C86:Q86"/>
+    <mergeCell ref="C78:Q78"/>
+    <mergeCell ref="C101:Q101"/>
+    <mergeCell ref="C92:Q92"/>
     <mergeCell ref="O15:Q15"/>
-    <mergeCell ref="C108:Q108"/>
     <mergeCell ref="B8:N8"/>
-    <mergeCell ref="C58:Q58"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="C104:Q104"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="F11:H15"/>
     <mergeCell ref="K13:L13"/>
+    <mergeCell ref="C88:Q88"/>
     <mergeCell ref="B10:N10"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="K18:M166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K18:M171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Passed,Failed,Pending,Not Executed"</formula1>
     </dataValidation>
-    <dataValidation sqref="O18:Q166" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O18:Q171" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"P,F,PE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>